<commit_message>
One wall stands on a property, so a claim is charged for one wall
Where a retaining wall is already there and vul finds it damaged, its
replacement is the whole of the wall cost and holds the landslide ground
as well. Where the property has no wall, or one vul finds undamaged, a
wall is invented for the ground instead. The two never both appear.

This replaces the one-metre-of-land-per-metre-of-wall allowance, which
was arbitrary and not monotonic, and drops the "new wall is never
smaller than the existing wall" rule, which is unreachable under it.
Across the pilot only three claims move.

The Repair cost tab is rebuilt around the asset -- landslide land, the
retaining wall, liquefaction, and the settlement -- GST-exclusive until
block D, and checks itself against the module to $0.00.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/report/loss/calc-walkthrough/loss-calculation-walkthrough.xlsx
+++ b/report/loss/calc-walkthrough/loss-calculation-walkthrough.xlsx
@@ -88,7 +88,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -103,6 +103,26 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0044546A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBE2D5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EDE3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7E6E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -123,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -153,12 +173,25 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1422,13 +1455,13 @@
         <v>0</v>
       </c>
       <c r="T10" s="7" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="U10" s="7" t="n">
         <v>28</v>
       </c>
       <c r="V10" s="8" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11">
@@ -1449,13 +1482,13 @@
         <v>0</v>
       </c>
       <c r="T11" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U11" s="7" t="n">
         <v>11</v>
       </c>
       <c r="V11" s="8" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12">
@@ -1475,7 +1508,7 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>13133909.54889522</v>
+        <v>13028775.83955245</v>
       </c>
     </row>
     <row r="14">
@@ -1520,7 +1553,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>20869279.22072987</v>
+        <v>20735243.5630001</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
@@ -1658,13 +1691,13 @@
         <v>0</v>
       </c>
       <c r="T21" s="7" t="n">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="U21" s="7" t="n">
         <v>42</v>
       </c>
       <c r="V21" s="8" t="n">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="22">
@@ -1677,13 +1710,13 @@
         <v>0</v>
       </c>
       <c r="T22" s="7" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="U22" s="7" t="n">
         <v>13</v>
       </c>
       <c r="V22" s="8" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="25">
@@ -1875,7 +1908,7 @@
         </is>
       </c>
       <c r="S37" s="13" t="n">
-        <v>1248769.097455249</v>
+        <v>1114733.43972548</v>
       </c>
     </row>
     <row r="38">
@@ -2227,7 +2260,7 @@
         <v/>
       </c>
       <c r="I15" s="22" t="n">
-        <v>62488.21263079525</v>
+        <v>35189.11647868678</v>
       </c>
       <c r="J15" s="21">
         <f>MIN(I15,H15)</f>
@@ -3218,1274 +3251,3184 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P36"/>
+  <dimension ref="A1:AO49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="15" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="17" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="10" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="16" customWidth="1" min="28" max="28"/>
+    <col width="10" customWidth="1" min="29" max="29"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
+    <col width="15" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="32" max="32"/>
+    <col width="16" customWidth="1" min="33" max="33"/>
+    <col width="15" customWidth="1" min="34" max="34"/>
+    <col width="13" customWidth="1" min="35" max="35"/>
+    <col width="13" customWidth="1" min="36" max="36"/>
+    <col width="14" customWidth="1" min="37" max="37"/>
+    <col width="13" customWidth="1" min="38" max="38"/>
+    <col width="12" customWidth="1" min="39" max="39"/>
+    <col width="15" customWidth="1" min="40" max="40"/>
+    <col width="15" customWidth="1" min="41" max="41"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Where the repair cost comes from</t>
+          <t>What is damaged, what it is worth, what repairing it costs</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Every line is an assumption, not a measurement. They are numbered so they can be referred to and decided one at a time.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="44" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
+          <t>One asset per block. Every dollar excludes GST until block D adds it once; the land values are market values, to which GST does not apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>A. Landslide land damage</t>
+        </is>
+      </c>
+      <c r="O4" s="26" t="inlineStr">
+        <is>
+          <t>B. Retaining wall damage</t>
+        </is>
+      </c>
+      <c r="V4" s="27" t="inlineStr">
+        <is>
+          <t>C. Liquefaction damage</t>
+        </is>
+      </c>
+      <c r="AC4" s="28" t="inlineStr">
+        <is>
+          <t>D. What is paid</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Claim</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>Wall size</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>Wall height (m)</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>Wall length (m)</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>Wall rate excl GST ($/m2)</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>1. Damaged wall replaced ($)</t>
-        </is>
-      </c>
-      <c r="G4" s="14" t="inlineStr">
-        <is>
-          <t>Landslide ground not covered by that wall (m2)</t>
-        </is>
-      </c>
-      <c r="H4" s="14" t="inlineStr">
-        <is>
-          <t>New wall size</t>
-        </is>
-      </c>
-      <c r="I4" s="14" t="inlineStr">
-        <is>
-          <t>New wall height (m)</t>
-        </is>
-      </c>
-      <c r="J4" s="14" t="inlineStr">
-        <is>
-          <t>New wall length (m)</t>
-        </is>
-      </c>
-      <c r="K4" s="14" t="inlineStr">
-        <is>
-          <t>2. New wall for landslide ground ($)</t>
-        </is>
-      </c>
-      <c r="L4" s="14" t="inlineStr">
-        <is>
-          <t>3. Spoil cleared ($)</t>
-        </is>
-      </c>
-      <c r="M4" s="14" t="inlineStr">
-        <is>
-          <t>4. Fees: consent, design, engineering, H&amp;S, PM, survey ($)</t>
-        </is>
-      </c>
-      <c r="N4" s="14" t="inlineStr">
-        <is>
-          <t>5. Liquefaction, Canterbury rates ($)</t>
-        </is>
-      </c>
-      <c r="O4" s="14" t="inlineStr">
-        <is>
-          <t>6. Culvert or bridge at sub-cap ($)</t>
-        </is>
-      </c>
-      <c r="P4" s="14" t="inlineStr">
-        <is>
-          <t>Total repair ($)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>03dc0301-b79a-4927-9dc7-cd7e95fc9aaf</t>
-        </is>
-      </c>
-      <c r="B5" s="25" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="C5" s="26" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="D5" s="27" t="n">
-        <v>6.313108289984361</v>
-      </c>
-      <c r="E5" s="28" t="n">
-        <v>798.8</v>
-      </c>
-      <c r="F5" s="29" t="n">
-        <v>12787.56131984668</v>
-      </c>
-      <c r="G5" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="25" t="inlineStr"/>
-      <c r="I5" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="29" t="n">
-        <v>325.0533090665411</v>
-      </c>
-      <c r="M5" s="29" t="n">
-        <v>6158.249999999999</v>
-      </c>
-      <c r="N5" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="30">
-        <f>F5+K5+L5+M5+N5+O5</f>
-        <v/>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Evacuated land (m2)</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>Inundated land (m2)</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>Imminent damage (m2) - not modelled yet</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>Total damaged land (m2)</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>Land rate ($/m2)</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>Value of damaged land ($)</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t>New RTW size</t>
+        </is>
+      </c>
+      <c r="I5" s="14" t="inlineStr">
+        <is>
+          <t>New RTW height (m)</t>
+        </is>
+      </c>
+      <c r="J5" s="14" t="inlineStr">
+        <is>
+          <t>New RTW length (m)</t>
+        </is>
+      </c>
+      <c r="K5" s="14" t="inlineStr">
+        <is>
+          <t>New RTW to hold it ($)</t>
+        </is>
+      </c>
+      <c r="L5" s="14" t="inlineStr">
+        <is>
+          <t>Spoil to clear (m3)</t>
+        </is>
+      </c>
+      <c r="M5" s="14" t="inlineStr">
+        <is>
+          <t>Spoil removal ($)</t>
+        </is>
+      </c>
+      <c r="N5" s="14" t="inlineStr">
+        <is>
+          <t>A. Landslide repair ($)</t>
+        </is>
+      </c>
+      <c r="O5" s="14" t="inlineStr">
+        <is>
+          <t>What damaged it</t>
+        </is>
+      </c>
+      <c r="P5" s="14" t="inlineStr">
+        <is>
+          <t>RTW size</t>
+        </is>
+      </c>
+      <c r="Q5" s="14" t="inlineStr">
+        <is>
+          <t>RTW height (m)</t>
+        </is>
+      </c>
+      <c r="R5" s="14" t="inlineStr">
+        <is>
+          <t>RTW length (m)</t>
+        </is>
+      </c>
+      <c r="S5" s="14" t="inlineStr">
+        <is>
+          <t>RTW rate ($/m2)</t>
+        </is>
+      </c>
+      <c r="T5" s="14" t="inlineStr">
+        <is>
+          <t>RTW undepreciated value ($)</t>
+        </is>
+      </c>
+      <c r="U5" s="14" t="inlineStr">
+        <is>
+          <t>B. RTW replacement ($)</t>
+        </is>
+      </c>
+      <c r="V5" s="14" t="inlineStr">
+        <is>
+          <t>Inundated land (m2) - not sent</t>
+        </is>
+      </c>
+      <c r="W5" s="14" t="inlineStr">
+        <is>
+          <t>Evacuated land, with lateral spreading (m2) - not sent</t>
+        </is>
+      </c>
+      <c r="X5" s="14" t="inlineStr">
+        <is>
+          <t>Liquefied land (m2)</t>
+        </is>
+      </c>
+      <c r="Y5" s="14" t="inlineStr">
+        <is>
+          <t>Total insured land (m2)</t>
+        </is>
+      </c>
+      <c r="Z5" s="14" t="inlineStr">
+        <is>
+          <t>Damage state</t>
+        </is>
+      </c>
+      <c r="AA5" s="14" t="inlineStr">
+        <is>
+          <t>Value of liquefied land ($)</t>
+        </is>
+      </c>
+      <c r="AB5" s="14" t="inlineStr">
+        <is>
+          <t>C. Liquefaction repair ($)</t>
+        </is>
+      </c>
+      <c r="AC5" s="14" t="inlineStr">
+        <is>
+          <t>Dwellings</t>
+        </is>
+      </c>
+      <c r="AD5" s="14" t="inlineStr">
+        <is>
+          <t>Professional fees ($)</t>
+        </is>
+      </c>
+      <c r="AE5" s="14" t="inlineStr">
+        <is>
+          <t>Total repair, excl GST ($)</t>
+        </is>
+      </c>
+      <c r="AF5" s="14" t="inlineStr">
+        <is>
+          <t>GST ($)</t>
+        </is>
+      </c>
+      <c r="AG5" s="14" t="inlineStr">
+        <is>
+          <t>Culvert or bridge at its sub-cap ($)</t>
+        </is>
+      </c>
+      <c r="AH5" s="14" t="inlineStr">
+        <is>
+          <t>Total repair, incl GST ($)</t>
+        </is>
+      </c>
+      <c r="AI5" s="14" t="inlineStr">
+        <is>
+          <t>Cap: land value ($)</t>
+        </is>
+      </c>
+      <c r="AJ5" s="14" t="inlineStr">
+        <is>
+          <t>Cap: RTW value ($)</t>
+        </is>
+      </c>
+      <c r="AK5" s="14" t="inlineStr">
+        <is>
+          <t>Land cover cap ($)</t>
+        </is>
+      </c>
+      <c r="AL5" s="14" t="inlineStr">
+        <is>
+          <t>Cost to pay ($)</t>
+        </is>
+      </c>
+      <c r="AM5" s="14" t="inlineStr">
+        <is>
+          <t>Excess ($)</t>
+        </is>
+      </c>
+      <c r="AN5" s="14" t="inlineStr">
+        <is>
+          <t>Settlement, incl GST ($)</t>
+        </is>
+      </c>
+      <c r="AO5" s="14" t="inlineStr">
+        <is>
+          <t>Settlement, excl GST ($)</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>331011f8-ce50-46ad-9aeb-03fffa6c8506</t>
-        </is>
-      </c>
-      <c r="B6" s="25" t="inlineStr">
-        <is>
-          <t>large</t>
-        </is>
-      </c>
-      <c r="C6" s="26" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="D6" s="27" t="n">
-        <v>8.159218973584622</v>
-      </c>
-      <c r="E6" s="28" t="n">
+          <t>03dc0301-b79a-4927-9dc7-cd7e95fc9aaf</t>
+        </is>
+      </c>
+      <c r="B6" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="29" t="n">
+        <v>3.994276433826656</v>
+      </c>
+      <c r="D6" s="29" t="n"/>
+      <c r="E6" s="29" t="n">
+        <v>3.994276433826656</v>
+      </c>
+      <c r="F6" s="30" t="n">
+        <v>906.9153731669335</v>
+      </c>
+      <c r="G6" s="31">
+        <f>MIN(E6,Calculation!$B$3)*F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="4" t="inlineStr"/>
+      <c r="I6" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="29" t="n">
+        <v>1.884367009081398</v>
+      </c>
+      <c r="M6" s="33" t="n">
+        <v>282.6550513622097</v>
+      </c>
+      <c r="N6" s="31">
+        <f>K6+M6</f>
+        <v/>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>shaking</t>
+        </is>
+      </c>
+      <c r="P6" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="Q6" s="32" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="R6" s="29" t="n">
+        <v>6.313108289984361</v>
+      </c>
+      <c r="S6" s="30" t="n">
         <v>798.8</v>
       </c>
-      <c r="F6" s="29" t="n">
-        <v>28444.36647868678</v>
-      </c>
-      <c r="G6" s="27" t="n">
-        <v>3.460588805527991</v>
-      </c>
-      <c r="H6" s="25" t="inlineStr">
-        <is>
-          <t>large</t>
-        </is>
-      </c>
-      <c r="I6" s="26" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="J6" s="27" t="n">
-        <v>8.159218973584622</v>
-      </c>
-      <c r="K6" s="29" t="n">
-        <v>27299.09615210847</v>
-      </c>
-      <c r="L6" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" s="29" t="n">
-        <v>6744.749999999999</v>
-      </c>
-      <c r="N6" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="30">
-        <f>F6+K6+L6+M6+N6+O6</f>
+      <c r="T6" s="33" t="n">
+        <v>8825.094078569136</v>
+      </c>
+      <c r="U6" s="33" t="n">
+        <v>11119.61853899711</v>
+      </c>
+      <c r="V6" s="29" t="n"/>
+      <c r="W6" s="29" t="n"/>
+      <c r="X6" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="29" t="n">
+        <v>159.4213451242771</v>
+      </c>
+      <c r="Z6" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="31">
+        <f>MIN(X6,Calculation!$B$3)*F6</f>
+        <v/>
+      </c>
+      <c r="AB6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD6" s="33" t="n">
+        <v>5355</v>
+      </c>
+      <c r="AE6" s="31">
+        <f>N6+U6+AB6+AD6</f>
+        <v/>
+      </c>
+      <c r="AF6" s="31">
+        <f>AE6*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH6" s="31">
+        <f>AE6+AF6+AG6</f>
+        <v/>
+      </c>
+      <c r="AI6" s="31">
+        <f>MAX(G6,AA6)</f>
+        <v/>
+      </c>
+      <c r="AJ6" s="31">
+        <f>MIN(T6*(1+Calculation!$B$9),Calculation!$B$4*AC6)</f>
+        <v/>
+      </c>
+      <c r="AK6" s="31">
+        <f>AI6+AJ6+AG6</f>
+        <v/>
+      </c>
+      <c r="AL6" s="31">
+        <f>MIN(AH6,AK6)</f>
+        <v/>
+      </c>
+      <c r="AM6" s="31">
+        <f>MIN(MAX(AL6*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL6&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN6" s="31">
+        <f>MAX(0,AL6-AM6)</f>
+        <v/>
+      </c>
+      <c r="AO6" s="31">
+        <f>AN6/(1+Calculation!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>36df7f1f-d454-4fd8-9751-1db3ad4e883a</t>
-        </is>
-      </c>
-      <c r="B7" s="25" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="C7" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="27" t="n">
-        <v>5.254910674327313</v>
-      </c>
-      <c r="H7" s="25" t="inlineStr">
-        <is>
-          <t>small</t>
-        </is>
-      </c>
-      <c r="I7" s="26" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J7" s="27" t="n">
-        <v>7.241885461988845</v>
-      </c>
-      <c r="K7" s="29" t="n">
-        <v>6320.839249637844</v>
+          <t>331011f8-ce50-46ad-9aeb-03fffa6c8506</t>
+        </is>
+      </c>
+      <c r="B7" s="29" t="n">
+        <v>11.61980777911261</v>
+      </c>
+      <c r="C7" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="29" t="n"/>
+      <c r="E7" s="29" t="n">
+        <v>11.61980777911261</v>
+      </c>
+      <c r="F7" s="30" t="n">
+        <v>875.2256394431051</v>
+      </c>
+      <c r="G7" s="31">
+        <f>MIN(E7,Calculation!$B$3)*F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="33" t="n">
+        <v>0</v>
       </c>
       <c r="L7" s="29" t="n">
-        <v>407.9292629771223</v>
-      </c>
-      <c r="M7" s="29" t="n">
-        <v>6451.499999999999</v>
-      </c>
-      <c r="N7" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" s="30">
-        <f>F7+K7+L7+M7+N7+O7</f>
+        <v>0</v>
+      </c>
+      <c r="M7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="31">
+        <f>K7+M7</f>
+        <v/>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>shaking + evacuated</t>
+        </is>
+      </c>
+      <c r="P7" s="4" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="Q7" s="32" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="R7" s="29" t="n">
+        <v>8.159218973584622</v>
+      </c>
+      <c r="S7" s="30" t="n">
+        <v>798.8</v>
+      </c>
+      <c r="T7" s="33" t="n">
+        <v>17923.35631927334</v>
+      </c>
+      <c r="U7" s="33" t="n">
+        <v>24734.2317205972</v>
+      </c>
+      <c r="V7" s="29" t="n"/>
+      <c r="W7" s="29" t="n"/>
+      <c r="X7" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="29" t="n">
+        <v>266.2914170356131</v>
+      </c>
+      <c r="Z7" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="31">
+        <f>MIN(X7,Calculation!$B$3)*F7</f>
+        <v/>
+      </c>
+      <c r="AB7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD7" s="33" t="n">
+        <v>5865</v>
+      </c>
+      <c r="AE7" s="31">
+        <f>N7+U7+AB7+AD7</f>
+        <v/>
+      </c>
+      <c r="AF7" s="31">
+        <f>AE7*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH7" s="31">
+        <f>AE7+AF7+AG7</f>
+        <v/>
+      </c>
+      <c r="AI7" s="31">
+        <f>MAX(G7,AA7)</f>
+        <v/>
+      </c>
+      <c r="AJ7" s="31">
+        <f>MIN(T7*(1+Calculation!$B$9),Calculation!$B$4*AC7)</f>
+        <v/>
+      </c>
+      <c r="AK7" s="31">
+        <f>AI7+AJ7+AG7</f>
+        <v/>
+      </c>
+      <c r="AL7" s="31">
+        <f>MIN(AH7,AK7)</f>
+        <v/>
+      </c>
+      <c r="AM7" s="31">
+        <f>MIN(MAX(AL7*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL7&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN7" s="31">
+        <f>MAX(0,AL7-AM7)</f>
+        <v/>
+      </c>
+      <c r="AO7" s="31">
+        <f>AN7/(1+Calculation!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>3c9cb87a-ae7d-4616-b2f0-ffff94a2930b</t>
-        </is>
-      </c>
-      <c r="B8" s="25" t="inlineStr">
+          <t>36df7f1f-d454-4fd8-9751-1db3ad4e883a</t>
+        </is>
+      </c>
+      <c r="B8" s="29" t="n">
+        <v>2.739921778496873</v>
+      </c>
+      <c r="C8" s="29" t="n">
+        <v>5.254910674327312</v>
+      </c>
+      <c r="D8" s="29" t="n"/>
+      <c r="E8" s="29" t="n">
+        <v>5.254910674327313</v>
+      </c>
+      <c r="F8" s="30" t="n">
+        <v>1033.806982141251</v>
+      </c>
+      <c r="G8" s="31">
+        <f>MIN(E8,Calculation!$B$3)*F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>small</t>
+        </is>
+      </c>
+      <c r="I8" s="32" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J8" s="29" t="n">
+        <v>7.241885461988845</v>
+      </c>
+      <c r="K8" s="33" t="n">
+        <v>5496.381956206821</v>
+      </c>
+      <c r="L8" s="29" t="n">
+        <v>2.364807321606506</v>
+      </c>
+      <c r="M8" s="33" t="n">
+        <v>354.7210982409759</v>
+      </c>
+      <c r="N8" s="31">
+        <f>K8+M8</f>
+        <v/>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>wall present, undamaged</t>
+        </is>
+      </c>
+      <c r="P8" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="C8" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="27" t="n">
-        <v>83.99693044062862</v>
-      </c>
-      <c r="H8" s="25" t="inlineStr">
-        <is>
-          <t>large</t>
-        </is>
-      </c>
-      <c r="I8" s="26" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="J8" s="27" t="n">
-        <v>16.96124457300522</v>
-      </c>
-      <c r="K8" s="29" t="n">
-        <v>56748.89324051</v>
-      </c>
-      <c r="L8" s="29" t="n">
-        <v>17369.30287275514</v>
-      </c>
-      <c r="M8" s="29" t="n">
-        <v>6744.749999999999</v>
-      </c>
-      <c r="N8" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" s="30">
-        <f>F8+K8+L8+M8+N8+O8</f>
+      <c r="Q8" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" s="29" t="n"/>
+      <c r="W8" s="29" t="n"/>
+      <c r="X8" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="29" t="n">
+        <v>420.2371467194171</v>
+      </c>
+      <c r="Z8" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" s="31">
+        <f>MIN(X8,Calculation!$B$3)*F8</f>
+        <v/>
+      </c>
+      <c r="AB8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC8" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD8" s="33" t="n">
+        <v>5610</v>
+      </c>
+      <c r="AE8" s="31">
+        <f>N8+U8+AB8+AD8</f>
+        <v/>
+      </c>
+      <c r="AF8" s="31">
+        <f>AE8*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH8" s="31">
+        <f>AE8+AF8+AG8</f>
+        <v/>
+      </c>
+      <c r="AI8" s="31">
+        <f>MAX(G8,AA8)</f>
+        <v/>
+      </c>
+      <c r="AJ8" s="31">
+        <f>MIN(T8*(1+Calculation!$B$9),Calculation!$B$4*AC8)</f>
+        <v/>
+      </c>
+      <c r="AK8" s="31">
+        <f>AI8+AJ8+AG8</f>
+        <v/>
+      </c>
+      <c r="AL8" s="31">
+        <f>MIN(AH8,AK8)</f>
+        <v/>
+      </c>
+      <c r="AM8" s="31">
+        <f>MIN(MAX(AL8*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL8&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN8" s="31">
+        <f>MAX(0,AL8-AM8)</f>
+        <v/>
+      </c>
+      <c r="AO8" s="31">
+        <f>AN8/(1+Calculation!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>06953c1e-a185-4880-a3e8-203ab7d4220a</t>
-        </is>
-      </c>
-      <c r="B9" s="25" t="inlineStr">
+          <t>3c9cb87a-ae7d-4616-b2f0-ffff94a2930b</t>
+        </is>
+      </c>
+      <c r="B9" s="29" t="n">
+        <v>4.81379863873295</v>
+      </c>
+      <c r="C9" s="29" t="n">
+        <v>83.99693044062863</v>
+      </c>
+      <c r="D9" s="29" t="n"/>
+      <c r="E9" s="29" t="n">
+        <v>83.99693044062862</v>
+      </c>
+      <c r="F9" s="30" t="n">
+        <v>952.5188914254333</v>
+      </c>
+      <c r="G9" s="31">
+        <f>MIN(E9,Calculation!$B$3)*F9</f>
+        <v/>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="I9" s="32" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="J9" s="29" t="n">
+        <v>16.96124457300522</v>
+      </c>
+      <c r="K9" s="33" t="n">
+        <v>49346.8636874</v>
+      </c>
+      <c r="L9" s="29" t="n">
+        <v>100.6916108565515</v>
+      </c>
+      <c r="M9" s="33" t="n">
+        <v>15103.74162848273</v>
+      </c>
+      <c r="N9" s="31">
+        <f>K9+M9</f>
+        <v/>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>no wall on the property</t>
+        </is>
+      </c>
+      <c r="P9" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="C9" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="27" t="n">
-        <v>31.56185795826037</v>
-      </c>
-      <c r="H9" s="25" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="I9" s="26" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="J9" s="27" t="n">
-        <v>11.94504348109692</v>
-      </c>
-      <c r="K9" s="29" t="n">
-        <v>26538.48795150091</v>
-      </c>
-      <c r="L9" s="29" t="n">
-        <v>1216.199339588118</v>
-      </c>
-      <c r="M9" s="29" t="n">
-        <v>7037.999999999999</v>
-      </c>
-      <c r="N9" s="29" t="n">
-        <v>230</v>
-      </c>
-      <c r="O9" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" s="30">
-        <f>F9+K9+L9+M9+N9+O9</f>
+      <c r="Q9" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" s="29" t="n"/>
+      <c r="W9" s="29" t="n"/>
+      <c r="X9" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" s="29" t="n">
+        <v>447.623704376365</v>
+      </c>
+      <c r="Z9" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA9" s="31">
+        <f>MIN(X9,Calculation!$B$3)*F9</f>
+        <v/>
+      </c>
+      <c r="AB9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC9" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD9" s="33" t="n">
+        <v>5865</v>
+      </c>
+      <c r="AE9" s="31">
+        <f>N9+U9+AB9+AD9</f>
+        <v/>
+      </c>
+      <c r="AF9" s="31">
+        <f>AE9*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH9" s="31">
+        <f>AE9+AF9+AG9</f>
+        <v/>
+      </c>
+      <c r="AI9" s="31">
+        <f>MAX(G9,AA9)</f>
+        <v/>
+      </c>
+      <c r="AJ9" s="31">
+        <f>MIN(T9*(1+Calculation!$B$9),Calculation!$B$4*AC9)</f>
+        <v/>
+      </c>
+      <c r="AK9" s="31">
+        <f>AI9+AJ9+AG9</f>
+        <v/>
+      </c>
+      <c r="AL9" s="31">
+        <f>MIN(AH9,AK9)</f>
+        <v/>
+      </c>
+      <c r="AM9" s="31">
+        <f>MIN(MAX(AL9*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL9&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN9" s="31">
+        <f>MAX(0,AL9-AM9)</f>
+        <v/>
+      </c>
+      <c r="AO9" s="31">
+        <f>AN9/(1+Calculation!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>0af1f540-21f2-4654-97ed-047e9a0d7e42</t>
-        </is>
-      </c>
-      <c r="B10" s="25" t="inlineStr">
+          <t>06953c1e-a185-4880-a3e8-203ab7d4220a</t>
+        </is>
+      </c>
+      <c r="B10" s="29" t="n">
+        <v>25.76580155440493</v>
+      </c>
+      <c r="C10" s="29" t="n">
+        <v>23.23198887690671</v>
+      </c>
+      <c r="D10" s="29" t="n"/>
+      <c r="E10" s="29" t="n">
+        <v>31.56185795826037</v>
+      </c>
+      <c r="F10" s="30" t="n">
+        <v>1215.255114101618</v>
+      </c>
+      <c r="G10" s="31">
+        <f>MIN(E10,Calculation!$B$3)*F10</f>
+        <v/>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="I10" s="32" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="J10" s="29" t="n">
+        <v>11.94504348109692</v>
+      </c>
+      <c r="K10" s="33" t="n">
+        <v>23076.9460447834</v>
+      </c>
+      <c r="L10" s="29" t="n">
+        <v>7.050430954134018</v>
+      </c>
+      <c r="M10" s="33" t="n">
+        <v>1057.564643120103</v>
+      </c>
+      <c r="N10" s="31">
+        <f>K10+M10</f>
+        <v/>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>no wall on the property</t>
+        </is>
+      </c>
+      <c r="P10" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="C10" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="27" t="n">
-        <v>5.903114465110614</v>
-      </c>
-      <c r="H10" s="25" t="inlineStr">
-        <is>
-          <t>small</t>
-        </is>
-      </c>
-      <c r="I10" s="26" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J10" s="27" t="n">
-        <v>7.436019343691363</v>
-      </c>
-      <c r="K10" s="29" t="n">
-        <v>6195.269718104418</v>
-      </c>
-      <c r="L10" s="29" t="n">
-        <v>93.17663389177265</v>
-      </c>
-      <c r="M10" s="29" t="n">
-        <v>6158.249999999999</v>
-      </c>
-      <c r="N10" s="29" t="n">
-        <v>575</v>
-      </c>
-      <c r="O10" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="30">
-        <f>F10+K10+L10+M10+N10+O10</f>
+      <c r="Q10" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" s="29" t="n"/>
+      <c r="W10" s="29" t="n"/>
+      <c r="X10" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="29" t="n">
+        <v>50447.22716690691</v>
+      </c>
+      <c r="Z10" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA10" s="31">
+        <f>MIN(X10,Calculation!$B$3)*F10</f>
+        <v/>
+      </c>
+      <c r="AB10" s="33" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC10" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD10" s="33" t="n">
+        <v>6120</v>
+      </c>
+      <c r="AE10" s="31">
+        <f>N10+U10+AB10+AD10</f>
+        <v/>
+      </c>
+      <c r="AF10" s="31">
+        <f>AE10*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG10" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH10" s="31">
+        <f>AE10+AF10+AG10</f>
+        <v/>
+      </c>
+      <c r="AI10" s="31">
+        <f>MAX(G10,AA10)</f>
+        <v/>
+      </c>
+      <c r="AJ10" s="31">
+        <f>MIN(T10*(1+Calculation!$B$9),Calculation!$B$4*AC10)</f>
+        <v/>
+      </c>
+      <c r="AK10" s="31">
+        <f>AI10+AJ10+AG10</f>
+        <v/>
+      </c>
+      <c r="AL10" s="31">
+        <f>MIN(AH10,AK10)</f>
+        <v/>
+      </c>
+      <c r="AM10" s="31">
+        <f>MIN(MAX(AL10*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL10&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN10" s="31">
+        <f>MAX(0,AL10-AM10)</f>
+        <v/>
+      </c>
+      <c r="AO10" s="31">
+        <f>AN10/(1+Calculation!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>0bc8522b-2de5-402b-b82e-ebb534151ee9</t>
-        </is>
-      </c>
-      <c r="B11" s="25" t="inlineStr">
+          <t>0af1f540-21f2-4654-97ed-047e9a0d7e42</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="n">
+        <v>5.636895421053411</v>
+      </c>
+      <c r="C11" s="29" t="n">
+        <v>3.183434007476635</v>
+      </c>
+      <c r="D11" s="29" t="n"/>
+      <c r="E11" s="29" t="n">
+        <v>5.903114465110614</v>
+      </c>
+      <c r="F11" s="30" t="n">
+        <v>1845.735003003669</v>
+      </c>
+      <c r="G11" s="31">
+        <f>MIN(E11,Calculation!$B$3)*F11</f>
+        <v/>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>small</t>
+        </is>
+      </c>
+      <c r="I11" s="32" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J11" s="29" t="n">
+        <v>7.436019343691363</v>
+      </c>
+      <c r="K11" s="33" t="n">
+        <v>5387.191059221233</v>
+      </c>
+      <c r="L11" s="29" t="n">
+        <v>0.5401543993725951</v>
+      </c>
+      <c r="M11" s="33" t="n">
+        <v>81.02315990588927</v>
+      </c>
+      <c r="N11" s="31">
+        <f>K11+M11</f>
+        <v/>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>no wall on the property</t>
+        </is>
+      </c>
+      <c r="P11" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="C11" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="27" t="n">
-        <v>15.48983220842302</v>
-      </c>
-      <c r="H11" s="25" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="I11" s="26" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="J11" s="27" t="n">
-        <v>9.565937873965719</v>
-      </c>
-      <c r="K11" s="29" t="n">
-        <v>17710.66017289853</v>
-      </c>
-      <c r="L11" s="29" t="n">
-        <v>693.2447350710288</v>
-      </c>
-      <c r="M11" s="29" t="n">
-        <v>5865</v>
-      </c>
-      <c r="N11" s="29" t="n">
-        <v>1725</v>
-      </c>
-      <c r="O11" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="30">
-        <f>F11+K11+L11+M11+N11+O11</f>
+      <c r="Q11" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" s="29" t="n"/>
+      <c r="W11" s="29" t="n"/>
+      <c r="X11" s="29" t="n">
+        <v>356.3788137462104</v>
+      </c>
+      <c r="Y11" s="29" t="n">
+        <v>356.3788137462104</v>
+      </c>
+      <c r="Z11" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA11" s="31">
+        <f>MIN(X11,Calculation!$B$3)*F11</f>
+        <v/>
+      </c>
+      <c r="AB11" s="33" t="n">
+        <v>500.0000000000001</v>
+      </c>
+      <c r="AC11" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD11" s="33" t="n">
+        <v>5355</v>
+      </c>
+      <c r="AE11" s="31">
+        <f>N11+U11+AB11+AD11</f>
+        <v/>
+      </c>
+      <c r="AF11" s="31">
+        <f>AE11*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG11" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH11" s="31">
+        <f>AE11+AF11+AG11</f>
+        <v/>
+      </c>
+      <c r="AI11" s="31">
+        <f>MAX(G11,AA11)</f>
+        <v/>
+      </c>
+      <c r="AJ11" s="31">
+        <f>MIN(T11*(1+Calculation!$B$9),Calculation!$B$4*AC11)</f>
+        <v/>
+      </c>
+      <c r="AK11" s="31">
+        <f>AI11+AJ11+AG11</f>
+        <v/>
+      </c>
+      <c r="AL11" s="31">
+        <f>MIN(AH11,AK11)</f>
+        <v/>
+      </c>
+      <c r="AM11" s="31">
+        <f>MIN(MAX(AL11*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL11&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN11" s="31">
+        <f>MAX(0,AL11-AM11)</f>
+        <v/>
+      </c>
+      <c r="AO11" s="31">
+        <f>AN11/(1+Calculation!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>0fb3766f-33f4-4b9d-95c4-74dbfc6876dd</t>
-        </is>
-      </c>
-      <c r="B12" s="25" t="inlineStr">
+          <t>0bc8522b-2de5-402b-b82e-ebb534151ee9</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="n">
+        <v>15.48983220842302</v>
+      </c>
+      <c r="C12" s="29" t="n">
+        <v>8.547847131838395</v>
+      </c>
+      <c r="D12" s="29" t="n"/>
+      <c r="E12" s="29" t="n">
+        <v>15.48983220842302</v>
+      </c>
+      <c r="F12" s="30" t="n">
+        <v>1750.105740634113</v>
+      </c>
+      <c r="G12" s="31">
+        <f>MIN(E12,Calculation!$B$3)*F12</f>
+        <v/>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="I12" s="32" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="J12" s="29" t="n">
+        <v>9.565937873965719</v>
+      </c>
+      <c r="K12" s="33" t="n">
+        <v>15400.57406339003</v>
+      </c>
+      <c r="L12" s="29" t="n">
+        <v>4.018810058382776</v>
+      </c>
+      <c r="M12" s="33" t="n">
+        <v>602.8215087574164</v>
+      </c>
+      <c r="N12" s="31">
+        <f>K12+M12</f>
+        <v/>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>no wall on the property</t>
+        </is>
+      </c>
+      <c r="P12" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="C12" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="27" t="n">
-        <v>34.1265011384118</v>
-      </c>
-      <c r="H12" s="25" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="I12" s="26" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="J12" s="27" t="n">
-        <v>12.26153752499035</v>
-      </c>
-      <c r="K12" s="29" t="n">
-        <v>23836.44170824372</v>
-      </c>
-      <c r="L12" s="29" t="n">
-        <v>1669.625992983824</v>
-      </c>
-      <c r="M12" s="29" t="n">
-        <v>6158.249999999999</v>
-      </c>
-      <c r="N12" s="29" t="n">
-        <v>230</v>
-      </c>
-      <c r="O12" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" s="30">
-        <f>F12+K12+L12+M12+N12+O12</f>
+      <c r="Q12" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" s="29" t="n"/>
+      <c r="W12" s="29" t="n"/>
+      <c r="X12" s="29" t="n">
+        <v>336.6041633096748</v>
+      </c>
+      <c r="Y12" s="29" t="n">
+        <v>336.6041633096748</v>
+      </c>
+      <c r="Z12" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA12" s="31">
+        <f>MIN(X12,Calculation!$B$3)*F12</f>
+        <v/>
+      </c>
+      <c r="AB12" s="33" t="n">
+        <v>1500</v>
+      </c>
+      <c r="AC12" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD12" s="33" t="n">
+        <v>5100</v>
+      </c>
+      <c r="AE12" s="31">
+        <f>N12+U12+AB12+AD12</f>
+        <v/>
+      </c>
+      <c r="AF12" s="31">
+        <f>AE12*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG12" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH12" s="31">
+        <f>AE12+AF12+AG12</f>
+        <v/>
+      </c>
+      <c r="AI12" s="31">
+        <f>MAX(G12,AA12)</f>
+        <v/>
+      </c>
+      <c r="AJ12" s="31">
+        <f>MIN(T12*(1+Calculation!$B$9),Calculation!$B$4*AC12)</f>
+        <v/>
+      </c>
+      <c r="AK12" s="31">
+        <f>AI12+AJ12+AG12</f>
+        <v/>
+      </c>
+      <c r="AL12" s="31">
+        <f>MIN(AH12,AK12)</f>
+        <v/>
+      </c>
+      <c r="AM12" s="31">
+        <f>MIN(MAX(AL12*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL12&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN12" s="31">
+        <f>MAX(0,AL12-AM12)</f>
+        <v/>
+      </c>
+      <c r="AO12" s="31">
+        <f>AN12/(1+Calculation!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>0035a155-c4d3-4860-80e0-6c17481b3d61</t>
-        </is>
-      </c>
-      <c r="B13" s="25" t="inlineStr">
-        <is>
-          <t>small</t>
-        </is>
-      </c>
-      <c r="C13" s="26" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D13" s="27" t="n">
-        <v>6.238939737591432</v>
-      </c>
-      <c r="E13" s="28" t="n">
-        <v>1224.08</v>
-      </c>
-      <c r="F13" s="29" t="n">
-        <v>7904.255001380601</v>
-      </c>
-      <c r="G13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="25" t="inlineStr"/>
-      <c r="I13" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="29" t="n">
-        <v>0</v>
+          <t>0fb3766f-33f4-4b9d-95c4-74dbfc6876dd</t>
+        </is>
+      </c>
+      <c r="B13" s="29" t="n">
+        <v>28.16598323933578</v>
+      </c>
+      <c r="C13" s="29" t="n">
+        <v>28.16598323933578</v>
+      </c>
+      <c r="D13" s="29" t="n"/>
+      <c r="E13" s="29" t="n">
+        <v>34.1265011384118</v>
+      </c>
+      <c r="F13" s="30" t="n">
+        <v>2173.314579577944</v>
+      </c>
+      <c r="G13" s="31">
+        <f>MIN(E13,Calculation!$B$3)*F13</f>
+        <v/>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="I13" s="32" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="J13" s="29" t="n">
+        <v>12.26153752499035</v>
+      </c>
+      <c r="K13" s="33" t="n">
+        <v>20727.3406158641</v>
       </c>
       <c r="L13" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="29" t="n">
-        <v>5865</v>
-      </c>
-      <c r="N13" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="30">
-        <f>F13+K13+L13+M13+N13+O13</f>
+        <v>9.678991263674343</v>
+      </c>
+      <c r="M13" s="33" t="n">
+        <v>1451.848689551151</v>
+      </c>
+      <c r="N13" s="31">
+        <f>K13+M13</f>
+        <v/>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>no wall on the property</t>
+        </is>
+      </c>
+      <c r="P13" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q13" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" s="29" t="n"/>
+      <c r="W13" s="29" t="n"/>
+      <c r="X13" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="29" t="n">
+        <v>836.0527260023529</v>
+      </c>
+      <c r="Z13" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA13" s="31">
+        <f>MIN(X13,Calculation!$B$3)*F13</f>
+        <v/>
+      </c>
+      <c r="AB13" s="33" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC13" s="35" t="n">
+        <v>9</v>
+      </c>
+      <c r="AD13" s="33" t="n">
+        <v>5355</v>
+      </c>
+      <c r="AE13" s="31">
+        <f>N13+U13+AB13+AD13</f>
+        <v/>
+      </c>
+      <c r="AF13" s="31">
+        <f>AE13*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH13" s="31">
+        <f>AE13+AF13+AG13</f>
+        <v/>
+      </c>
+      <c r="AI13" s="31">
+        <f>MAX(G13,AA13)</f>
+        <v/>
+      </c>
+      <c r="AJ13" s="31">
+        <f>MIN(T13*(1+Calculation!$B$9),Calculation!$B$4*AC13)</f>
+        <v/>
+      </c>
+      <c r="AK13" s="31">
+        <f>AI13+AJ13+AG13</f>
+        <v/>
+      </c>
+      <c r="AL13" s="31">
+        <f>MIN(AH13,AK13)</f>
+        <v/>
+      </c>
+      <c r="AM13" s="31">
+        <f>MIN(MAX(AL13*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL13&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN13" s="31">
+        <f>MAX(0,AL13-AM13)</f>
+        <v/>
+      </c>
+      <c r="AO13" s="31">
+        <f>AN13/(1+Calculation!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>00745333-cf86-4178-8cf6-cd6f9d7d5cbd</t>
-        </is>
-      </c>
-      <c r="B14" s="25" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="C14" s="26" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="D14" s="27" t="n">
-        <v>8.711899422777982</v>
-      </c>
-      <c r="E14" s="28" t="n">
-        <v>798.8</v>
-      </c>
-      <c r="F14" s="29" t="n">
-        <v>17646.44973029384</v>
-      </c>
-      <c r="G14" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="25" t="inlineStr"/>
-      <c r="I14" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" s="29" t="n">
+          <t>0035a155-c4d3-4860-80e0-6c17481b3d61</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="29" t="n"/>
+      <c r="E14" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="30" t="n">
+        <v>1125.800303002638</v>
+      </c>
+      <c r="G14" s="31">
+        <f>MIN(E14,Calculation!$B$3)*F14</f>
+        <v/>
+      </c>
+      <c r="H14" s="4" t="inlineStr"/>
+      <c r="I14" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="33" t="n">
         <v>0</v>
       </c>
       <c r="L14" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="M14" s="29" t="n">
-        <v>6158.249999999999</v>
-      </c>
-      <c r="N14" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" s="30">
-        <f>F14+K14+L14+M14+N14+O14</f>
+      <c r="M14" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="31">
+        <f>K14+M14</f>
+        <v/>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>shaking</t>
+        </is>
+      </c>
+      <c r="P14" s="4" t="inlineStr">
+        <is>
+          <t>small</t>
+        </is>
+      </c>
+      <c r="Q14" s="32" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="R14" s="29" t="n">
+        <v>6.238939737591432</v>
+      </c>
+      <c r="S14" s="30" t="n">
+        <v>1224.08</v>
+      </c>
+      <c r="T14" s="33" t="n">
+        <v>5727.72101549319</v>
+      </c>
+      <c r="U14" s="33" t="n">
+        <v>6873.265218591828</v>
+      </c>
+      <c r="V14" s="29" t="n"/>
+      <c r="W14" s="29" t="n"/>
+      <c r="X14" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="29" t="n">
+        <v>155.6974761971898</v>
+      </c>
+      <c r="Z14" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="31">
+        <f>MIN(X14,Calculation!$B$3)*F14</f>
+        <v/>
+      </c>
+      <c r="AB14" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC14" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD14" s="33" t="n">
+        <v>5100</v>
+      </c>
+      <c r="AE14" s="31">
+        <f>N14+U14+AB14+AD14</f>
+        <v/>
+      </c>
+      <c r="AF14" s="31">
+        <f>AE14*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG14" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH14" s="31">
+        <f>AE14+AF14+AG14</f>
+        <v/>
+      </c>
+      <c r="AI14" s="31">
+        <f>MAX(G14,AA14)</f>
+        <v/>
+      </c>
+      <c r="AJ14" s="31">
+        <f>MIN(T14*(1+Calculation!$B$9),Calculation!$B$4*AC14)</f>
+        <v/>
+      </c>
+      <c r="AK14" s="31">
+        <f>AI14+AJ14+AG14</f>
+        <v/>
+      </c>
+      <c r="AL14" s="31">
+        <f>MIN(AH14,AK14)</f>
+        <v/>
+      </c>
+      <c r="AM14" s="31">
+        <f>MIN(MAX(AL14*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL14&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN14" s="31">
+        <f>MAX(0,AL14-AM14)</f>
+        <v/>
+      </c>
+      <c r="AO14" s="31">
+        <f>AN14/(1+Calculation!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>00a83d76-9c9c-4d92-8d56-b16f1336cabb</t>
-        </is>
-      </c>
-      <c r="B15" s="25" t="inlineStr">
+          <t>00745333-cf86-4178-8cf6-cd6f9d7d5cbd</t>
+        </is>
+      </c>
+      <c r="B15" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="29" t="n"/>
+      <c r="E15" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="30" t="n">
+        <v>990.5549772618464</v>
+      </c>
+      <c r="G15" s="31">
+        <f>MIN(E15,Calculation!$B$3)*F15</f>
+        <v/>
+      </c>
+      <c r="H15" s="4" t="inlineStr"/>
+      <c r="I15" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="31">
+        <f>K15+M15</f>
+        <v/>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>shaking</t>
+        </is>
+      </c>
+      <c r="P15" s="4" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="C15" s="26" t="n">
+      <c r="Q15" s="32" t="n">
         <v>1.75</v>
       </c>
-      <c r="D15" s="27" t="n">
-        <v>9.70437961684674</v>
-      </c>
-      <c r="E15" s="28" t="n">
-        <v>643.1900000000001</v>
-      </c>
-      <c r="F15" s="29" t="n">
-        <v>16581.23524278052</v>
-      </c>
-      <c r="G15" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="25" t="inlineStr"/>
-      <c r="I15" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="29" t="n">
-        <v>6451.499999999999</v>
-      </c>
-      <c r="N15" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" s="30">
-        <f>F15+K15+L15+M15+N15+O15</f>
+      <c r="R15" s="29" t="n">
+        <v>8.711899422777982</v>
+      </c>
+      <c r="S15" s="30" t="n">
+        <v>798.8</v>
+      </c>
+      <c r="T15" s="33" t="n">
+        <v>12178.36420310134</v>
+      </c>
+      <c r="U15" s="33" t="n">
+        <v>15344.73889590769</v>
+      </c>
+      <c r="V15" s="29" t="n"/>
+      <c r="W15" s="29" t="n"/>
+      <c r="X15" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="29" t="n">
+        <v>303.5887662103974</v>
+      </c>
+      <c r="Z15" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA15" s="31">
+        <f>MIN(X15,Calculation!$B$3)*F15</f>
+        <v/>
+      </c>
+      <c r="AB15" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC15" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD15" s="33" t="n">
+        <v>5355</v>
+      </c>
+      <c r="AE15" s="31">
+        <f>N15+U15+AB15+AD15</f>
+        <v/>
+      </c>
+      <c r="AF15" s="31">
+        <f>AE15*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG15" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH15" s="31">
+        <f>AE15+AF15+AG15</f>
+        <v/>
+      </c>
+      <c r="AI15" s="31">
+        <f>MAX(G15,AA15)</f>
+        <v/>
+      </c>
+      <c r="AJ15" s="31">
+        <f>MIN(T15*(1+Calculation!$B$9),Calculation!$B$4*AC15)</f>
+        <v/>
+      </c>
+      <c r="AK15" s="31">
+        <f>AI15+AJ15+AG15</f>
+        <v/>
+      </c>
+      <c r="AL15" s="31">
+        <f>MIN(AH15,AK15)</f>
+        <v/>
+      </c>
+      <c r="AM15" s="31">
+        <f>MIN(MAX(AL15*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL15&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN15" s="31">
+        <f>MAX(0,AL15-AM15)</f>
+        <v/>
+      </c>
+      <c r="AO15" s="31">
+        <f>AN15/(1+Calculation!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>01b4d137-3ac2-408b-9de3-c572fc374ef4</t>
-        </is>
-      </c>
-      <c r="B16" s="25" t="inlineStr">
+          <t>00a83d76-9c9c-4d92-8d56-b16f1336cabb</t>
+        </is>
+      </c>
+      <c r="B16" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="29" t="n"/>
+      <c r="E16" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="30" t="n">
+        <v>909.0124673749219</v>
+      </c>
+      <c r="G16" s="31">
+        <f>MIN(E16,Calculation!$B$3)*F16</f>
+        <v/>
+      </c>
+      <c r="H16" s="4" t="inlineStr"/>
+      <c r="I16" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="31">
+        <f>K16+M16</f>
+        <v/>
+      </c>
+      <c r="O16" s="4" t="inlineStr">
+        <is>
+          <t>shaking</t>
+        </is>
+      </c>
+      <c r="P16" s="4" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="C16" s="26" t="n">
+      <c r="Q16" s="32" t="n">
         <v>1.75</v>
       </c>
-      <c r="D16" s="27" t="n">
-        <v>10.86560963197419</v>
-      </c>
-      <c r="E16" s="28" t="n">
-        <v>879.87</v>
-      </c>
-      <c r="F16" s="29" t="n">
-        <v>24242.59144831398</v>
-      </c>
-      <c r="G16" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="25" t="inlineStr"/>
-      <c r="I16" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="29" t="n">
-        <v>6158.249999999999</v>
-      </c>
-      <c r="N16" s="29" t="n">
-        <v>575</v>
-      </c>
-      <c r="O16" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="30">
-        <f>F16+K16+L16+M16+N16+O16</f>
+      <c r="R16" s="29" t="n">
+        <v>9.70437961684674</v>
+      </c>
+      <c r="S16" s="30" t="n">
+        <v>643.1900000000001</v>
+      </c>
+      <c r="T16" s="33" t="n">
+        <v>10923.0798700794</v>
+      </c>
+      <c r="U16" s="33" t="n">
+        <v>14418.4654285048</v>
+      </c>
+      <c r="V16" s="29" t="n"/>
+      <c r="W16" s="29" t="n"/>
+      <c r="X16" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="29" t="n">
+        <v>376.6999349914819</v>
+      </c>
+      <c r="Z16" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA16" s="31">
+        <f>MIN(X16,Calculation!$B$3)*F16</f>
+        <v/>
+      </c>
+      <c r="AB16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC16" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD16" s="33" t="n">
+        <v>5610</v>
+      </c>
+      <c r="AE16" s="31">
+        <f>N16+U16+AB16+AD16</f>
+        <v/>
+      </c>
+      <c r="AF16" s="31">
+        <f>AE16*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH16" s="31">
+        <f>AE16+AF16+AG16</f>
+        <v/>
+      </c>
+      <c r="AI16" s="31">
+        <f>MAX(G16,AA16)</f>
+        <v/>
+      </c>
+      <c r="AJ16" s="31">
+        <f>MIN(T16*(1+Calculation!$B$9),Calculation!$B$4*AC16)</f>
+        <v/>
+      </c>
+      <c r="AK16" s="31">
+        <f>AI16+AJ16+AG16</f>
+        <v/>
+      </c>
+      <c r="AL16" s="31">
+        <f>MIN(AH16,AK16)</f>
+        <v/>
+      </c>
+      <c r="AM16" s="31">
+        <f>MIN(MAX(AL16*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL16&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN16" s="31">
+        <f>MAX(0,AL16-AM16)</f>
+        <v/>
+      </c>
+      <c r="AO16" s="31">
+        <f>AN16/(1+Calculation!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>0017e6f7-95ee-4d2a-8bff-569d98d70ec8</t>
-        </is>
-      </c>
-      <c r="B17" s="25" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="C17" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="25" t="inlineStr"/>
-      <c r="I17" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" s="29" t="n">
+          <t>01b4d137-3ac2-408b-9de3-c572fc374ef4</t>
+        </is>
+      </c>
+      <c r="B17" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="29" t="n"/>
+      <c r="E17" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="30" t="n">
+        <v>1669.724652985133</v>
+      </c>
+      <c r="G17" s="31">
+        <f>MIN(E17,Calculation!$B$3)*F17</f>
+        <v/>
+      </c>
+      <c r="H17" s="4" t="inlineStr"/>
+      <c r="I17" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="33" t="n">
         <v>0</v>
       </c>
       <c r="L17" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="M17" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" s="29" t="n">
-        <v>4600</v>
-      </c>
-      <c r="O17" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" s="30">
-        <f>F17+K17+L17+M17+N17+O17</f>
+      <c r="M17" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="31">
+        <f>K17+M17</f>
+        <v/>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>shaking</t>
+        </is>
+      </c>
+      <c r="P17" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="Q17" s="32" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="R17" s="29" t="n">
+        <v>10.86560963197419</v>
+      </c>
+      <c r="S17" s="30" t="n">
+        <v>879.87</v>
+      </c>
+      <c r="T17" s="33" t="n">
+        <v>16730.56690704899</v>
+      </c>
+      <c r="U17" s="33" t="n">
+        <v>21080.51430288172</v>
+      </c>
+      <c r="V17" s="29" t="n"/>
+      <c r="W17" s="29" t="n"/>
+      <c r="X17" s="29" t="n">
+        <v>472.2458906978015</v>
+      </c>
+      <c r="Y17" s="29" t="n">
+        <v>472.2458906978015</v>
+      </c>
+      <c r="Z17" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA17" s="31">
+        <f>MIN(X17,Calculation!$B$3)*F17</f>
+        <v/>
+      </c>
+      <c r="AB17" s="33" t="n">
+        <v>500.0000000000001</v>
+      </c>
+      <c r="AC17" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD17" s="33" t="n">
+        <v>5355</v>
+      </c>
+      <c r="AE17" s="31">
+        <f>N17+U17+AB17+AD17</f>
+        <v/>
+      </c>
+      <c r="AF17" s="31">
+        <f>AE17*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG17" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH17" s="31">
+        <f>AE17+AF17+AG17</f>
+        <v/>
+      </c>
+      <c r="AI17" s="31">
+        <f>MAX(G17,AA17)</f>
+        <v/>
+      </c>
+      <c r="AJ17" s="31">
+        <f>MIN(T17*(1+Calculation!$B$9),Calculation!$B$4*AC17)</f>
+        <v/>
+      </c>
+      <c r="AK17" s="31">
+        <f>AI17+AJ17+AG17</f>
+        <v/>
+      </c>
+      <c r="AL17" s="31">
+        <f>MIN(AH17,AK17)</f>
+        <v/>
+      </c>
+      <c r="AM17" s="31">
+        <f>MIN(MAX(AL17*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL17&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN17" s="31">
+        <f>MAX(0,AL17-AM17)</f>
+        <v/>
+      </c>
+      <c r="AO17" s="31">
+        <f>AN17/(1+Calculation!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>00191a75-aed6-4265-a79b-faa275f0040c</t>
-        </is>
-      </c>
-      <c r="B18" s="25" t="inlineStr">
+          <t>0017e6f7-95ee-4d2a-8bff-569d98d70ec8</t>
+        </is>
+      </c>
+      <c r="B18" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="29" t="n"/>
+      <c r="E18" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="30" t="n">
+        <v>1908.027810002991</v>
+      </c>
+      <c r="G18" s="31">
+        <f>MIN(E18,Calculation!$B$3)*F18</f>
+        <v/>
+      </c>
+      <c r="H18" s="4" t="inlineStr"/>
+      <c r="I18" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="31">
+        <f>K18+M18</f>
+        <v/>
+      </c>
+      <c r="O18" s="4" t="inlineStr">
+        <is>
+          <t>no wall on the property</t>
+        </is>
+      </c>
+      <c r="P18" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="C18" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="25" t="inlineStr"/>
-      <c r="I18" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" s="29" t="n">
-        <v>1725</v>
-      </c>
-      <c r="O18" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P18" s="30">
-        <f>F18+K18+L18+M18+N18+O18</f>
+      <c r="Q18" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U18" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" s="29" t="n"/>
+      <c r="W18" s="29" t="n"/>
+      <c r="X18" s="29" t="n">
+        <v>2824.033182987902</v>
+      </c>
+      <c r="Y18" s="29" t="n">
+        <v>2824.033182987902</v>
+      </c>
+      <c r="Z18" s="34" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA18" s="31">
+        <f>MIN(X18,Calculation!$B$3)*F18</f>
+        <v/>
+      </c>
+      <c r="AB18" s="33" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AC18" s="35" t="n">
+        <v>29</v>
+      </c>
+      <c r="AD18" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE18" s="31">
+        <f>N18+U18+AB18+AD18</f>
+        <v/>
+      </c>
+      <c r="AF18" s="31">
+        <f>AE18*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG18" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH18" s="31">
+        <f>AE18+AF18+AG18</f>
+        <v/>
+      </c>
+      <c r="AI18" s="31">
+        <f>MAX(G18,AA18)</f>
+        <v/>
+      </c>
+      <c r="AJ18" s="31">
+        <f>MIN(T18*(1+Calculation!$B$9),Calculation!$B$4*AC18)</f>
+        <v/>
+      </c>
+      <c r="AK18" s="31">
+        <f>AI18+AJ18+AG18</f>
+        <v/>
+      </c>
+      <c r="AL18" s="31">
+        <f>MIN(AH18,AK18)</f>
+        <v/>
+      </c>
+      <c r="AM18" s="31">
+        <f>MIN(MAX(AL18*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL18&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN18" s="31">
+        <f>MAX(0,AL18-AM18)</f>
+        <v/>
+      </c>
+      <c r="AO18" s="31">
+        <f>AN18/(1+Calculation!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>001e2f9c-9846-4a4d-aff2-1de9e7b091c7</t>
-        </is>
-      </c>
-      <c r="B19" s="25" t="inlineStr">
+          <t>00191a75-aed6-4265-a79b-faa275f0040c</t>
+        </is>
+      </c>
+      <c r="B19" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="29" t="n"/>
+      <c r="E19" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="30" t="n">
+        <v>1891.519728815266</v>
+      </c>
+      <c r="G19" s="31">
+        <f>MIN(E19,Calculation!$B$3)*F19</f>
+        <v/>
+      </c>
+      <c r="H19" s="4" t="inlineStr"/>
+      <c r="I19" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="31">
+        <f>K19+M19</f>
+        <v/>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>no wall on the property</t>
+        </is>
+      </c>
+      <c r="P19" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="C19" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="25" t="inlineStr"/>
-      <c r="I19" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" s="29" t="n">
-        <v>1725</v>
-      </c>
-      <c r="O19" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" s="30">
-        <f>F19+K19+L19+M19+N19+O19</f>
+      <c r="Q19" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V19" s="29" t="n"/>
+      <c r="W19" s="29" t="n"/>
+      <c r="X19" s="29" t="n">
+        <v>286.0372101473818</v>
+      </c>
+      <c r="Y19" s="29" t="n">
+        <v>286.0372101473818</v>
+      </c>
+      <c r="Z19" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA19" s="31">
+        <f>MIN(X19,Calculation!$B$3)*F19</f>
+        <v/>
+      </c>
+      <c r="AB19" s="33" t="n">
+        <v>1500</v>
+      </c>
+      <c r="AC19" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD19" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE19" s="31">
+        <f>N19+U19+AB19+AD19</f>
+        <v/>
+      </c>
+      <c r="AF19" s="31">
+        <f>AE19*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG19" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH19" s="31">
+        <f>AE19+AF19+AG19</f>
+        <v/>
+      </c>
+      <c r="AI19" s="31">
+        <f>MAX(G19,AA19)</f>
+        <v/>
+      </c>
+      <c r="AJ19" s="31">
+        <f>MIN(T19*(1+Calculation!$B$9),Calculation!$B$4*AC19)</f>
+        <v/>
+      </c>
+      <c r="AK19" s="31">
+        <f>AI19+AJ19+AG19</f>
+        <v/>
+      </c>
+      <c r="AL19" s="31">
+        <f>MIN(AH19,AK19)</f>
+        <v/>
+      </c>
+      <c r="AM19" s="31">
+        <f>MIN(MAX(AL19*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL19&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN19" s="31">
+        <f>MAX(0,AL19-AM19)</f>
+        <v/>
+      </c>
+      <c r="AO19" s="31">
+        <f>AN19/(1+Calculation!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>0055aa62-333d-49e8-8a1b-4277448835ed</t>
-        </is>
-      </c>
-      <c r="B20" s="25" t="inlineStr">
+          <t>001e2f9c-9846-4a4d-aff2-1de9e7b091c7</t>
+        </is>
+      </c>
+      <c r="B20" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="29" t="n"/>
+      <c r="E20" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="30" t="n">
+        <v>1603.475556633135</v>
+      </c>
+      <c r="G20" s="31">
+        <f>MIN(E20,Calculation!$B$3)*F20</f>
+        <v/>
+      </c>
+      <c r="H20" s="4" t="inlineStr"/>
+      <c r="I20" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="31">
+        <f>K20+M20</f>
+        <v/>
+      </c>
+      <c r="O20" s="4" t="inlineStr">
+        <is>
+          <t>no wall on the property</t>
+        </is>
+      </c>
+      <c r="P20" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="C20" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="25" t="inlineStr"/>
-      <c r="I20" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" s="29" t="n">
-        <v>575</v>
-      </c>
-      <c r="O20" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" s="30">
-        <f>F20+K20+L20+M20+N20+O20</f>
+      <c r="Q20" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U20" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" s="29" t="n"/>
+      <c r="W20" s="29" t="n"/>
+      <c r="X20" s="29" t="n">
+        <v>192.3987560767283</v>
+      </c>
+      <c r="Y20" s="29" t="n">
+        <v>192.3987560767283</v>
+      </c>
+      <c r="Z20" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA20" s="31">
+        <f>MIN(X20,Calculation!$B$3)*F20</f>
+        <v/>
+      </c>
+      <c r="AB20" s="33" t="n">
+        <v>1500</v>
+      </c>
+      <c r="AC20" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD20" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE20" s="31">
+        <f>N20+U20+AB20+AD20</f>
+        <v/>
+      </c>
+      <c r="AF20" s="31">
+        <f>AE20*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG20" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH20" s="31">
+        <f>AE20+AF20+AG20</f>
+        <v/>
+      </c>
+      <c r="AI20" s="31">
+        <f>MAX(G20,AA20)</f>
+        <v/>
+      </c>
+      <c r="AJ20" s="31">
+        <f>MIN(T20*(1+Calculation!$B$9),Calculation!$B$4*AC20)</f>
+        <v/>
+      </c>
+      <c r="AK20" s="31">
+        <f>AI20+AJ20+AG20</f>
+        <v/>
+      </c>
+      <c r="AL20" s="31">
+        <f>MIN(AH20,AK20)</f>
+        <v/>
+      </c>
+      <c r="AM20" s="31">
+        <f>MIN(MAX(AL20*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL20&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN20" s="31">
+        <f>MAX(0,AL20-AM20)</f>
+        <v/>
+      </c>
+      <c r="AO20" s="31">
+        <f>AN20/(1+Calculation!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>002e15d9-b27f-4a99-b94d-703b11215eab</t>
-        </is>
-      </c>
-      <c r="B21" s="25" t="inlineStr">
+          <t>0055aa62-333d-49e8-8a1b-4277448835ed</t>
+        </is>
+      </c>
+      <c r="B21" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="29" t="n"/>
+      <c r="E21" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="30" t="n">
+        <v>1832.043468426193</v>
+      </c>
+      <c r="G21" s="31">
+        <f>MIN(E21,Calculation!$B$3)*F21</f>
+        <v/>
+      </c>
+      <c r="H21" s="4" t="inlineStr"/>
+      <c r="I21" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="31">
+        <f>K21+M21</f>
+        <v/>
+      </c>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>no wall on the property</t>
+        </is>
+      </c>
+      <c r="P21" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="C21" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="25" t="inlineStr"/>
-      <c r="I21" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" s="30">
-        <f>F21+K21+L21+M21+N21+O21</f>
+      <c r="Q21" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T21" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V21" s="29" t="n"/>
+      <c r="W21" s="29" t="n"/>
+      <c r="X21" s="29" t="n">
+        <v>212.7684182341731</v>
+      </c>
+      <c r="Y21" s="29" t="n">
+        <v>212.7684182341731</v>
+      </c>
+      <c r="Z21" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA21" s="31">
+        <f>MIN(X21,Calculation!$B$3)*F21</f>
+        <v/>
+      </c>
+      <c r="AB21" s="33" t="n">
+        <v>500.0000000000001</v>
+      </c>
+      <c r="AC21" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD21" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE21" s="31">
+        <f>N21+U21+AB21+AD21</f>
+        <v/>
+      </c>
+      <c r="AF21" s="31">
+        <f>AE21*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG21" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH21" s="31">
+        <f>AE21+AF21+AG21</f>
+        <v/>
+      </c>
+      <c r="AI21" s="31">
+        <f>MAX(G21,AA21)</f>
+        <v/>
+      </c>
+      <c r="AJ21" s="31">
+        <f>MIN(T21*(1+Calculation!$B$9),Calculation!$B$4*AC21)</f>
+        <v/>
+      </c>
+      <c r="AK21" s="31">
+        <f>AI21+AJ21+AG21</f>
+        <v/>
+      </c>
+      <c r="AL21" s="31">
+        <f>MIN(AH21,AK21)</f>
+        <v/>
+      </c>
+      <c r="AM21" s="31">
+        <f>MIN(MAX(AL21*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL21&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN21" s="31">
+        <f>MAX(0,AL21-AM21)</f>
+        <v/>
+      </c>
+      <c r="AO21" s="31">
+        <f>AN21/(1+Calculation!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>0120d782-7901-4838-9ae8-012ec8626771</t>
-        </is>
-      </c>
-      <c r="B22" s="25" t="inlineStr">
+          <t>002e15d9-b27f-4a99-b94d-703b11215eab</t>
+        </is>
+      </c>
+      <c r="B22" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="29" t="n"/>
+      <c r="E22" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="30" t="n">
+        <v>816.216729440072</v>
+      </c>
+      <c r="G22" s="31">
+        <f>MIN(E22,Calculation!$B$3)*F22</f>
+        <v/>
+      </c>
+      <c r="H22" s="4" t="inlineStr"/>
+      <c r="I22" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="31">
+        <f>K22+M22</f>
+        <v/>
+      </c>
+      <c r="O22" s="4" t="inlineStr">
+        <is>
+          <t>no wall on the property</t>
+        </is>
+      </c>
+      <c r="P22" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="C22" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" s="25" t="inlineStr"/>
-      <c r="I22" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M22" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" s="29" t="n">
-        <v>230</v>
-      </c>
-      <c r="O22" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" s="30">
-        <f>F22+K22+L22+M22+N22+O22</f>
+      <c r="Q22" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T22" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U22" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V22" s="29" t="n"/>
+      <c r="W22" s="29" t="n"/>
+      <c r="X22" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y22" s="29" t="n">
+        <v>252.3366353326147</v>
+      </c>
+      <c r="Z22" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA22" s="31">
+        <f>MIN(X22,Calculation!$B$3)*F22</f>
+        <v/>
+      </c>
+      <c r="AB22" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="35" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD22" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE22" s="31">
+        <f>N22+U22+AB22+AD22</f>
+        <v/>
+      </c>
+      <c r="AF22" s="31">
+        <f>AE22*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG22" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH22" s="31">
+        <f>AE22+AF22+AG22</f>
+        <v/>
+      </c>
+      <c r="AI22" s="31">
+        <f>MAX(G22,AA22)</f>
+        <v/>
+      </c>
+      <c r="AJ22" s="31">
+        <f>MIN(T22*(1+Calculation!$B$9),Calculation!$B$4*AC22)</f>
+        <v/>
+      </c>
+      <c r="AK22" s="31">
+        <f>AI22+AJ22+AG22</f>
+        <v/>
+      </c>
+      <c r="AL22" s="31">
+        <f>MIN(AH22,AK22)</f>
+        <v/>
+      </c>
+      <c r="AM22" s="31">
+        <f>MIN(MAX(AL22*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL22&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN22" s="31">
+        <f>MAX(0,AL22-AM22)</f>
+        <v/>
+      </c>
+      <c r="AO22" s="31">
+        <f>AN22/(1+Calculation!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>012c131a-dea5-4ece-8e66-1e6f0f73959e</t>
-        </is>
-      </c>
-      <c r="B23" s="25" t="inlineStr">
+          <t>0120d782-7901-4838-9ae8-012ec8626771</t>
+        </is>
+      </c>
+      <c r="B23" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="29" t="n"/>
+      <c r="E23" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="30" t="n">
+        <v>1691.829478035887</v>
+      </c>
+      <c r="G23" s="31">
+        <f>MIN(E23,Calculation!$B$3)*F23</f>
+        <v/>
+      </c>
+      <c r="H23" s="4" t="inlineStr"/>
+      <c r="I23" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="31">
+        <f>K23+M23</f>
+        <v/>
+      </c>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t>no wall on the property</t>
+        </is>
+      </c>
+      <c r="P23" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="C23" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="25" t="inlineStr"/>
-      <c r="I23" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" s="29" t="n">
-        <v>230</v>
-      </c>
-      <c r="O23" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" s="30">
-        <f>F23+K23+L23+M23+N23+O23</f>
+      <c r="Q23" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T23" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U23" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V23" s="29" t="n"/>
+      <c r="W23" s="29" t="n"/>
+      <c r="X23" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y23" s="29" t="n">
+        <v>413.2027308032251</v>
+      </c>
+      <c r="Z23" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA23" s="31">
+        <f>MIN(X23,Calculation!$B$3)*F23</f>
+        <v/>
+      </c>
+      <c r="AB23" s="33" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC23" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD23" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE23" s="31">
+        <f>N23+U23+AB23+AD23</f>
+        <v/>
+      </c>
+      <c r="AF23" s="31">
+        <f>AE23*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG23" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH23" s="31">
+        <f>AE23+AF23+AG23</f>
+        <v/>
+      </c>
+      <c r="AI23" s="31">
+        <f>MAX(G23,AA23)</f>
+        <v/>
+      </c>
+      <c r="AJ23" s="31">
+        <f>MIN(T23*(1+Calculation!$B$9),Calculation!$B$4*AC23)</f>
+        <v/>
+      </c>
+      <c r="AK23" s="31">
+        <f>AI23+AJ23+AG23</f>
+        <v/>
+      </c>
+      <c r="AL23" s="31">
+        <f>MIN(AH23,AK23)</f>
+        <v/>
+      </c>
+      <c r="AM23" s="31">
+        <f>MIN(MAX(AL23*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL23&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN23" s="31">
+        <f>MAX(0,AL23-AM23)</f>
+        <v/>
+      </c>
+      <c r="AO23" s="31">
+        <f>AN23/(1+Calculation!$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
+          <t>012c131a-dea5-4ece-8e66-1e6f0f73959e</t>
+        </is>
+      </c>
+      <c r="B24" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="29" t="n"/>
+      <c r="E24" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="30" t="n">
+        <v>1982.685871232275</v>
+      </c>
+      <c r="G24" s="31">
+        <f>MIN(E24,Calculation!$B$3)*F24</f>
+        <v/>
+      </c>
+      <c r="H24" s="4" t="inlineStr"/>
+      <c r="I24" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="31">
+        <f>K24+M24</f>
+        <v/>
+      </c>
+      <c r="O24" s="4" t="inlineStr">
+        <is>
+          <t>no wall on the property</t>
+        </is>
+      </c>
+      <c r="P24" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q24" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S24" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T24" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U24" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V24" s="29" t="n"/>
+      <c r="W24" s="29" t="n"/>
+      <c r="X24" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y24" s="29" t="n">
+        <v>185.6254252003966</v>
+      </c>
+      <c r="Z24" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA24" s="31">
+        <f>MIN(X24,Calculation!$B$3)*F24</f>
+        <v/>
+      </c>
+      <c r="AB24" s="33" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC24" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD24" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE24" s="31">
+        <f>N24+U24+AB24+AD24</f>
+        <v/>
+      </c>
+      <c r="AF24" s="31">
+        <f>AE24*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG24" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH24" s="31">
+        <f>AE24+AF24+AG24</f>
+        <v/>
+      </c>
+      <c r="AI24" s="31">
+        <f>MAX(G24,AA24)</f>
+        <v/>
+      </c>
+      <c r="AJ24" s="31">
+        <f>MIN(T24*(1+Calculation!$B$9),Calculation!$B$4*AC24)</f>
+        <v/>
+      </c>
+      <c r="AK24" s="31">
+        <f>AI24+AJ24+AG24</f>
+        <v/>
+      </c>
+      <c r="AL24" s="31">
+        <f>MIN(AH24,AK24)</f>
+        <v/>
+      </c>
+      <c r="AM24" s="31">
+        <f>MIN(MAX(AL24*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL24&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN24" s="31">
+        <f>MAX(0,AL24-AM24)</f>
+        <v/>
+      </c>
+      <c r="AO24" s="31">
+        <f>AN24/(1+Calculation!$B$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
           <t>015ac9d8-763d-4df5-b585-423b129c132f</t>
         </is>
       </c>
-      <c r="B24" s="25" t="inlineStr">
+      <c r="B25" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="29" t="n"/>
+      <c r="E25" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="30" t="n">
+        <v>1772.056809778281</v>
+      </c>
+      <c r="G25" s="31">
+        <f>MIN(E25,Calculation!$B$3)*F25</f>
+        <v/>
+      </c>
+      <c r="H25" s="4" t="inlineStr"/>
+      <c r="I25" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="31">
+        <f>K25+M25</f>
+        <v/>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t>no wall on the property</t>
+        </is>
+      </c>
+      <c r="P25" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="C24" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="25" t="inlineStr"/>
-      <c r="I24" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" s="29" t="n">
-        <v>230</v>
-      </c>
-      <c r="O24" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" s="30">
-        <f>F24+K24+L24+M24+N24+O24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="31" t="inlineStr"/>
+      <c r="Q25" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T25" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U25" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V25" s="29" t="n"/>
+      <c r="W25" s="29" t="n"/>
+      <c r="X25" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y25" s="29" t="n">
+        <v>345.7075018575658</v>
+      </c>
+      <c r="Z25" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA25" s="31">
+        <f>MIN(X25,Calculation!$B$3)*F25</f>
+        <v/>
+      </c>
+      <c r="AB25" s="33" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC25" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD25" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE25" s="31">
+        <f>N25+U25+AB25+AD25</f>
+        <v/>
+      </c>
+      <c r="AF25" s="31">
+        <f>AE25*Calculation!$B$9</f>
+        <v/>
+      </c>
+      <c r="AG25" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH25" s="31">
+        <f>AE25+AF25+AG25</f>
+        <v/>
+      </c>
+      <c r="AI25" s="31">
+        <f>MAX(G25,AA25)</f>
+        <v/>
+      </c>
+      <c r="AJ25" s="31">
+        <f>MIN(T25*(1+Calculation!$B$9),Calculation!$B$4*AC25)</f>
+        <v/>
+      </c>
+      <c r="AK25" s="31">
+        <f>AI25+AJ25+AG25</f>
+        <v/>
+      </c>
+      <c r="AL25" s="31">
+        <f>MIN(AH25,AK25)</f>
+        <v/>
+      </c>
+      <c r="AM25" s="31">
+        <f>MIN(MAX(AL25*Calculation!$B$5,Calculation!$B$6),Calculation!$B$7)*(AL25&gt;0)</f>
+        <v/>
+      </c>
+      <c r="AN25" s="31">
+        <f>MAX(0,AL25-AM25)</f>
+        <v/>
+      </c>
+      <c r="AO25" s="31">
+        <f>AN25/(1+Calculation!$B$9)</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="32" t="inlineStr">
-        <is>
-          <t>Assumptions behind each column, to be confirmed:</t>
-        </is>
-      </c>
+      <c r="A28" s="36" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="31" t="inlineStr">
-        <is>
-          <t>1. Nothing says which of the tool's 29 construction types a wall is, so 30% are priced as Reinforced Concrete and the rest take one of four timber pole rates, drawn by hashing the wall id. The repair carries the site multiplier and a 20% allowance for the replacement being a better wall than the one that failed; the undepreciated value carries neither.</t>
+      <c r="A29" s="37" t="inlineStr">
+        <is>
+          <t>How to read this tab</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="31" t="inlineStr">
-        <is>
-          <t>2. A damaged wall is assumed to reinstate one metre of land for every metre of its length. Landslide ground beyond that gets a wall invented for it, sized by the uncovered area and the deposit volume, its length twice its depth plus 2 m at each end and never under 5 m. NOTE the uncovered area is the LANDSLIDE area only - liquefied ground is not remediated by a wall.</t>
+      <c r="A30" s="36" t="inlineStr">
+        <is>
+          <t>Each of the first three blocks is one asset, and asks the same four questions about it: what is it, what is it worth, what would repairing it cost, and what does it contribute. Block D turns the three answers into one settlement. Every dollar is GST-exclusive until block D adds GST once, on the row marked 'GST'.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="31" t="inlineStr">
-        <is>
-          <t>3. Spoil is cleared at the costing tool's own rate, 'Clear site: Load, cart and tip material', $150 per cubic metre excluding GST. The same volume also sets the earthworks rating, which is worth watching for a double count.</t>
+      <c r="A31" s="36" t="inlineStr">
+        <is>
+          <t>The land values are the exception and are not GST-exclusive, because a market value is not a GST-bearing price. The Act caps cover at the market value of the damaged land, and the repair bill NHC pays carries GST, so the two sides of MIN(repair, cap) are compared on the GST-inclusive basis. Whether that is the intended reading is still open (Q-14).</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="31" t="inlineStr">
-        <is>
-          <t>4. The six professional fees from the tool's fee table, $5,100 excluding GST, charged once on a claim that involves a wall and added before the site multiplier so a difficult site costs more to design as well as to build. Mileage is excluded, and they never reach the undepreciated value.</t>
-        </is>
-      </c>
+      <c r="A32" s="36" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="31" t="inlineStr">
-        <is>
-          <t>5. Canterbury settled costs per property, $200 to $4,000 by damage state. 2010/2011 dollars, grossed up for GST but NOT inflated. They exclude ILV and IFV, so they are the minor-damage tier only.</t>
+      <c r="A33" s="37" t="inlineStr">
+        <is>
+          <t>Empty columns, and why</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="31" t="inlineStr">
-        <is>
-          <t>6. Nothing prices a culvert or bridge, so a damaged one is assumed to exceed its sub-cap and is settled at the limit.</t>
+      <c r="A34" s="36" t="inlineStr">
+        <is>
+          <t>Imminent damage (block A) is not modelled yet. The agreed method is a second polygon of similar size centred on the same failure, its extra ground taken upslope to a new headscarp, with only the newly evacuated area counting. It belongs to vul and is calibrated off the claims reports.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="31" t="inlineStr"/>
+      <c r="A35" s="36" t="inlineStr">
+        <is>
+          <t>The three liquefaction extents (block C) are empty because vul sends liquefaction as a damage state with no footprint at all. Lateral spreading is being modelled as a magnification of the probability of states 4 to 6 near waterways, which moves a property's state rather than drawing an area -- so these columns may never be fillable in the form the heading implies.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="31" t="inlineStr">
-        <is>
-          <t>The three site ratings that mark up a wall's cost - construction access, earthworks and constructability - are proxied off driveway length, inundated volume and ground slope. All bands are invented. Together they can move a wall cost by at most 30%.</t>
+      <c r="A36" s="36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="37" t="inlineStr">
+        <is>
+          <t>Assumptions behind each figure, to be confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="36" t="inlineStr">
+        <is>
+          <t>A1. One wall stands on a property, so a claim is charged for one wall. Where a retaining wall is already there it is taken to be damaged and is replaced, and that replacement in block B is the whole of the wall cost -- block A is empty. Where there is no wall, one is invented to hold the ground and block B is empty. The two never both appear (decided 2026-09-29).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="36" t="inlineStr">
+        <is>
+          <t>A2. An invented wall is sized on the total damaged land -- the union of the evacuated and inundated footprints -- and on the deposit volume where an inundated depth gives one. Its length is twice the failure's depth plus 2 m at each end, never under 5 m. It is a remediation cost, not an asset, so it never reaches the cap: a wall that did not exist has no undepreciated value to contribute.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="36" t="inlineStr">
+        <is>
+          <t>A3. Spoil is cleared at the costing tool's own rate, 'Clear site: Load, cart and tip material', $150 per cubic metre excluding GST. The same volume also sets the earthworks rating, which is worth watching for a double count.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="36" t="inlineStr">
+        <is>
+          <t>B1. A wall already on the property is replaced rather than repaired: partial repair is about 1% of cases and is not modelled. Where the claim also has landslide ground, this replacement holds it, and no second wall is priced in block A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="36" t="inlineStr">
+        <is>
+          <t>B2. Nothing says which of the tool's 29 construction types a wall is, so 30% are priced as Reinforced Concrete and the rest take one of four timber pole rates, drawn by hashing the wall id. The replacement carries the site multiplier and a 20% allowance for being built to a better standard than the one that failed; the undepreciated value carries neither, which is the whole of the difference between them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="36" t="inlineStr">
+        <is>
+          <t>C1. Canterbury settled costs per property, $200 to $4,000 by damage state, in 2010/2011 dollars and NOT yet inflated. They exclude ILV and IFV, so they are the minor-damage tier only. The cap the state is compared against is the land rate over the whole insured area, because that is the scope those rates are per-property against.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="36" t="inlineStr">
+        <is>
+          <t>D1. The six professional fees from the tool's fee table, $5,100 excluding GST, charged once on a claim that involves a wall and added before the site multiplier, so a difficult site costs more to design as well as to build. Mileage is excluded, and they never reach the undepreciated value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="36" t="inlineStr">
+        <is>
+          <t>D2. Nothing prices a culvert or bridge, so a damaged one is assumed to exceed its sub-cap and is settled at the limit -- which is why it appears on both sides and carries no GST line of its own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="36" t="inlineStr">
+        <is>
+          <t>D3. The cap's land value is the LARGER of block A's and block C's, not their sum. A section that both liquefied and was buried is one piece of damaged ground, and adding the two would value some of it twice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="36" t="inlineStr">
+        <is>
+          <t>D4. MIN(repair, cap) is taken once, at claim level, over every asset together. The excess is a share of what would otherwise be paid, floored and capped, and a claim paid nothing is charged nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="36" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="36" t="inlineStr">
+        <is>
+          <t>The three site ratings that mark up a wall's cost -- construction access, earthworks and constructability -- are proxied off driveway length, inundated volume and ground slope. All bands are invented. Together they can move a wall cost by at most 30%.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="V4:AB4"/>
+    <mergeCell ref="O4:U4"/>
+    <mergeCell ref="B4:N4"/>
+    <mergeCell ref="AC4:AO4"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Read the loss tables per exposure world (T-66)
The loss module asked for the four vul tables by earthquake only,
through the deprecated loss_input_path, which always read world 0. Steps
0 and 1, the calculation walkthrough and the viewer now read through
world_loss_input_path with a WORLD_IDS setting beside REALISATION_IDS,
and loss_input_path and its tests are deleted.

The land cover cap and settlement files and the viewer CSV carry the
world in their names (-w000-r000) and a world_id column, so a second
world no longer overwrites the first. Re-run over the pilot: caps and
settlements written for world 0, step 1's cap agrees with step 0's.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/report/loss/calc-walkthrough/loss-calculation-walkthrough.xlsx
+++ b/report/loss/calc-walkthrough/loss-calculation-walkthrough.xlsx
@@ -1292,16 +1292,16 @@
         </is>
       </c>
       <c r="S4" s="7" t="n">
-        <v>664</v>
+        <v>479</v>
       </c>
       <c r="T4" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="U4" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="V4" s="8" t="n">
-        <v>664</v>
+        <v>486</v>
       </c>
     </row>
     <row r="5">
@@ -1319,16 +1319,16 @@
         </is>
       </c>
       <c r="S5" s="7" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="T5" s="7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U5" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="V5" s="8" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6">
@@ -1346,16 +1346,16 @@
         </is>
       </c>
       <c r="S6" s="7" t="n">
-        <v>582</v>
+        <v>513</v>
       </c>
       <c r="T6" s="7" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="U6" s="7" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="V6" s="8" t="n">
-        <v>584</v>
+        <v>552</v>
       </c>
     </row>
     <row r="7">
@@ -1373,16 +1373,16 @@
         </is>
       </c>
       <c r="S7" s="7" t="n">
-        <v>178</v>
+        <v>23</v>
       </c>
       <c r="T7" s="7" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="U7" s="7" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="V7" s="8" t="n">
-        <v>202</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8">
@@ -1395,13 +1395,13 @@
         <v>0</v>
       </c>
       <c r="T8" s="7" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="U8" s="7" t="n">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="V8" s="8" t="n">
-        <v>51</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9">
@@ -1414,13 +1414,13 @@
         <v>0</v>
       </c>
       <c r="T9" s="7" t="n">
-        <v>278</v>
+        <v>193</v>
       </c>
       <c r="U9" s="7" t="n">
-        <v>73</v>
+        <v>241</v>
       </c>
       <c r="V9" s="8" t="n">
-        <v>351</v>
+        <v>434</v>
       </c>
     </row>
     <row r="10">
@@ -1438,13 +1438,13 @@
         <v>0</v>
       </c>
       <c r="T10" s="7" t="n">
-        <v>93</v>
+        <v>440</v>
       </c>
       <c r="U10" s="7" t="n">
-        <v>30</v>
+        <v>254</v>
       </c>
       <c r="V10" s="8" t="n">
-        <v>123</v>
+        <v>694</v>
       </c>
     </row>
     <row r="11">
@@ -1454,7 +1454,7 @@
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>4388</v>
+        <v>4295</v>
       </c>
       <c r="R11" s="4" t="inlineStr">
         <is>
@@ -1465,13 +1465,13 @@
         <v>0</v>
       </c>
       <c r="T11" s="7" t="n">
-        <v>5</v>
+        <v>787</v>
       </c>
       <c r="U11" s="7" t="n">
-        <v>11</v>
+        <v>179</v>
       </c>
       <c r="V11" s="8" t="n">
-        <v>16</v>
+        <v>966</v>
       </c>
     </row>
     <row r="12">
@@ -1481,7 +1481,7 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>2031</v>
+        <v>3316</v>
       </c>
     </row>
     <row r="13">
@@ -1491,7 +1491,7 @@
         </is>
       </c>
       <c r="B13" s="11" t="n">
-        <v>13682686.79732165</v>
+        <v>163784521.6857729</v>
       </c>
     </row>
     <row r="14">
@@ -1501,7 +1501,7 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>1225</v>
+        <v>25034.20091420833</v>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
@@ -1536,7 +1536,7 @@
         </is>
       </c>
       <c r="B15" s="12" t="n">
-        <v>20846758.63635068</v>
+        <v>192656282.7048594</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
@@ -1544,7 +1544,7 @@
         </is>
       </c>
       <c r="S15" s="7" t="n">
-        <v>635</v>
+        <v>456</v>
       </c>
       <c r="T15" s="7" t="n">
         <v>0</v>
@@ -1553,7 +1553,7 @@
         <v>0</v>
       </c>
       <c r="V15" s="8" t="n">
-        <v>635</v>
+        <v>456</v>
       </c>
     </row>
     <row r="16">
@@ -1563,7 +1563,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>11</v>
+        <v>526</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="S16" s="7" t="n">
-        <v>849</v>
+        <v>576</v>
       </c>
       <c r="T16" s="7" t="n">
         <v>0</v>
@@ -1580,7 +1580,7 @@
         <v>0</v>
       </c>
       <c r="V16" s="8" t="n">
-        <v>849</v>
+        <v>576</v>
       </c>
     </row>
     <row r="17">
@@ -1590,7 +1590,7 @@
         </is>
       </c>
       <c r="S17" s="7" t="n">
-        <v>581</v>
+        <v>560</v>
       </c>
       <c r="T17" s="7" t="n">
         <v>0</v>
@@ -1599,7 +1599,7 @@
         <v>0</v>
       </c>
       <c r="V17" s="8" t="n">
-        <v>581</v>
+        <v>560</v>
       </c>
     </row>
     <row r="18">
@@ -1614,7 +1614,7 @@
         </is>
       </c>
       <c r="S18" s="7" t="n">
-        <v>286</v>
+        <v>59</v>
       </c>
       <c r="T18" s="7" t="n">
         <v>0</v>
@@ -1623,7 +1623,7 @@
         <v>0</v>
       </c>
       <c r="V18" s="8" t="n">
-        <v>286</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19">
@@ -1636,13 +1636,13 @@
         <v>0</v>
       </c>
       <c r="T19" s="7" t="n">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="U19" s="7" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="V19" s="8" t="n">
-        <v>4</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20">
@@ -1655,13 +1655,13 @@
         <v>0</v>
       </c>
       <c r="T20" s="7" t="n">
-        <v>149</v>
+        <v>208</v>
       </c>
       <c r="U20" s="7" t="n">
-        <v>83</v>
+        <v>266</v>
       </c>
       <c r="V20" s="8" t="n">
-        <v>232</v>
+        <v>474</v>
       </c>
     </row>
     <row r="21">
@@ -1674,13 +1674,13 @@
         <v>0</v>
       </c>
       <c r="T21" s="7" t="n">
-        <v>245</v>
+        <v>479</v>
       </c>
       <c r="U21" s="7" t="n">
-        <v>35</v>
+        <v>275</v>
       </c>
       <c r="V21" s="8" t="n">
-        <v>280</v>
+        <v>754</v>
       </c>
     </row>
     <row r="22">
@@ -1693,13 +1693,13 @@
         <v>0</v>
       </c>
       <c r="T22" s="7" t="n">
-        <v>39</v>
+        <v>812</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>13</v>
+        <v>188</v>
       </c>
       <c r="V22" s="8" t="n">
-        <v>52</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="25">
@@ -1736,16 +1736,16 @@
         </is>
       </c>
       <c r="S26" s="7" t="n">
-        <v>1</v>
+        <v>580</v>
       </c>
       <c r="T26" s="7" t="n">
-        <v>434</v>
+        <v>744</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>33</v>
+        <v>334</v>
       </c>
       <c r="V26" s="8" t="n">
-        <v>468</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="27">
@@ -1755,16 +1755,16 @@
         </is>
       </c>
       <c r="S27" s="7" t="n">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="T27" s="7" t="n">
-        <v>1</v>
+        <v>518</v>
       </c>
       <c r="U27" s="7" t="n">
-        <v>14</v>
+        <v>183</v>
       </c>
       <c r="V27" s="8" t="n">
-        <v>119</v>
+        <v>817</v>
       </c>
     </row>
     <row r="28">
@@ -1774,16 +1774,16 @@
         </is>
       </c>
       <c r="S28" s="7" t="n">
-        <v>660</v>
+        <v>312</v>
       </c>
       <c r="T28" s="7" t="n">
-        <v>0</v>
+        <v>249</v>
       </c>
       <c r="U28" s="7" t="n">
-        <v>38</v>
+        <v>164</v>
       </c>
       <c r="V28" s="8" t="n">
-        <v>698</v>
+        <v>725</v>
       </c>
     </row>
     <row r="29">
@@ -1793,16 +1793,16 @@
         </is>
       </c>
       <c r="S29" s="7" t="n">
-        <v>537</v>
+        <v>151</v>
       </c>
       <c r="T29" s="7" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="V29" s="8" t="n">
-        <v>566</v>
+        <v>211</v>
       </c>
     </row>
     <row r="30">
@@ -1812,16 +1812,16 @@
         </is>
       </c>
       <c r="S30" s="7" t="n">
-        <v>221</v>
+        <v>23</v>
       </c>
       <c r="T30" s="7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="V30" s="8" t="n">
-        <v>230</v>
+        <v>39</v>
       </c>
     </row>
     <row r="31">
@@ -1831,16 +1831,16 @@
         </is>
       </c>
       <c r="S31" s="7" t="n">
-        <v>128</v>
+        <v>9</v>
       </c>
       <c r="T31" s="7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U31" s="7" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="V31" s="8" t="n">
-        <v>131</v>
+        <v>23</v>
       </c>
     </row>
     <row r="32">
@@ -1850,16 +1850,16 @@
         </is>
       </c>
       <c r="S32" s="7" t="n">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="T32" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U32" s="7" t="n">
         <v>7</v>
       </c>
       <c r="V32" s="8" t="n">
-        <v>72</v>
+        <v>12</v>
       </c>
     </row>
     <row r="35">
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="S36" s="12" t="n">
-        <v>12733196.81184714</v>
+        <v>115002451.3169562</v>
       </c>
     </row>
     <row r="37">
@@ -1891,7 +1891,7 @@
         </is>
       </c>
       <c r="S37" s="12" t="n">
-        <v>1125271.660897423</v>
+        <v>39351835.66461074</v>
       </c>
     </row>
     <row r="38">
@@ -1901,7 +1901,7 @@
         </is>
       </c>
       <c r="S38" s="12" t="n">
-        <v>492687.6636061204</v>
+        <v>21546748.72329243</v>
       </c>
     </row>
     <row r="39">
@@ -1911,7 +1911,7 @@
         </is>
       </c>
       <c r="S39" s="12" t="n">
-        <v>3562987.5</v>
+        <v>14362212</v>
       </c>
     </row>
     <row r="40">
@@ -1921,7 +1921,7 @@
         </is>
       </c>
       <c r="S40" s="12" t="n">
-        <v>2932615</v>
+        <v>2393035</v>
       </c>
     </row>
     <row r="41">
@@ -2100,7 +2100,7 @@
       <c r="B13" s="15" t="inlineStr"/>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>whole insured area where liquefied, else the slip</t>
+          <t>MAX(liquefied land, the slip)</t>
         </is>
       </c>
       <c r="D13" s="15" t="inlineStr"/>
@@ -2144,24 +2144,24 @@
     <row r="14">
       <c r="A14" s="16" t="inlineStr">
         <is>
-          <t>03dc0301-b79a-4927-9dc7-cd7e95fc9aaf</t>
+          <t>018d3ae8-debe-4c14-8b06-2870c121761e</t>
         </is>
       </c>
       <c r="B14" s="17" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="18" t="n">
-        <v>3.994276433826656</v>
+        <v>0.9297514124773443</v>
       </c>
       <c r="D14" s="19" t="n">
-        <v>906.9153731669335</v>
+        <v>1643.133438311629</v>
       </c>
       <c r="E14" s="20">
         <f>MIN(C14,$B$3)*D14</f>
         <v/>
       </c>
       <c r="F14" s="21" t="n">
-        <v>9461.383582592764</v>
+        <v>0</v>
       </c>
       <c r="G14" s="20">
         <f>MIN(F14,$B$4*B14)</f>
@@ -2172,7 +2172,7 @@
         <v/>
       </c>
       <c r="I14" s="21" t="n">
-        <v>19373.92514052142</v>
+        <v>9435.581258178707</v>
       </c>
       <c r="J14" s="20">
         <f>MIN(I14,H14)</f>
@@ -2195,24 +2195,24 @@
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>331011f8-ce50-46ad-9aeb-03fffa6c8506</t>
+          <t>01f4c88f-c20c-48a2-a1e1-c3994510daa1</t>
         </is>
       </c>
       <c r="B15" s="17" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="18" t="n">
-        <v>11.61980777911261</v>
+        <v>1.642472856392285</v>
       </c>
       <c r="D15" s="19" t="n">
-        <v>875.2256394431051</v>
+        <v>1610.224150599341</v>
       </c>
       <c r="E15" s="20">
         <f>MIN(C15,$B$3)*D15</f>
         <v/>
       </c>
       <c r="F15" s="21" t="n">
-        <v>20611.85976716434</v>
+        <v>2584.395515180543</v>
       </c>
       <c r="G15" s="20">
         <f>MIN(F15,$B$4*B15)</f>
@@ -2223,7 +2223,7 @@
         <v/>
       </c>
       <c r="I15" s="21" t="n">
-        <v>37495.31597494504</v>
+        <v>10353.50230353578</v>
       </c>
       <c r="J15" s="20">
         <f>MIN(I15,H15)</f>
@@ -2246,17 +2246,17 @@
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>36df7f1f-d454-4fd8-9751-1db3ad4e883a</t>
+          <t>01f97a58-c26c-468a-b02f-b75858b5575b</t>
         </is>
       </c>
       <c r="B16" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16" s="18" t="n">
-        <v>5.254910674327313</v>
+        <v>10.88333781855425</v>
       </c>
       <c r="D16" s="19" t="n">
-        <v>1033.806982141251</v>
+        <v>1991.793188542959</v>
       </c>
       <c r="E16" s="20">
         <f>MIN(C16,$B$3)*D16</f>
@@ -2274,7 +2274,7 @@
         <v/>
       </c>
       <c r="I16" s="21" t="n">
-        <v>12162.45787424981</v>
+        <v>22664.27702712718</v>
       </c>
       <c r="J16" s="20">
         <f>MIN(I16,H16)</f>
@@ -2297,17 +2297,17 @@
     <row r="17">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t>3c9cb87a-ae7d-4616-b2f0-ffff94a2930b</t>
+          <t>02d672fd-0ee8-4e6a-9e86-e092694dc40f</t>
         </is>
       </c>
       <c r="B17" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="C17" s="18" t="n">
-        <v>83.99693044062862</v>
-      </c>
       <c r="D17" s="19" t="n">
-        <v>952.5188914254333</v>
+        <v>2002.415796489682</v>
       </c>
       <c r="E17" s="20">
         <f>MIN(C17,$B$3)*D17</f>
@@ -2325,7 +2325,7 @@
         <v/>
       </c>
       <c r="I17" s="21" t="n">
-        <v>83243.71444099226</v>
+        <v>9814.463408065891</v>
       </c>
       <c r="J17" s="20">
         <f>MIN(I17,H17)</f>
@@ -2348,17 +2348,17 @@
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>06953c1e-a185-4880-a3e8-203ab7d4220a</t>
+          <t>001e2f9c-9846-4a4d-aff2-1de9e7b091c7</t>
         </is>
       </c>
       <c r="B18" s="17" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C18" s="18" t="n">
-        <v>31.56185795826037</v>
+        <v>75.53717854302793</v>
       </c>
       <c r="D18" s="19" t="n">
-        <v>1215.255114101618</v>
+        <v>2915.070027166179</v>
       </c>
       <c r="E18" s="20">
         <f>MIN(C18,$B$3)*D18</f>
@@ -2376,7 +2376,7 @@
         <v/>
       </c>
       <c r="I18" s="21" t="n">
-        <v>34262.93647754864</v>
+        <v>24195.58752938664</v>
       </c>
       <c r="J18" s="20">
         <f>MIN(I18,H18)</f>
@@ -2399,17 +2399,17 @@
     <row r="19">
       <c r="A19" s="16" t="inlineStr">
         <is>
-          <t>0af1f540-21f2-4654-97ed-047e9a0d7e42</t>
+          <t>00224faa-3597-401e-b493-559fc185861b</t>
         </is>
       </c>
       <c r="B19" s="17" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="18" t="n">
-        <v>356.3788137462104</v>
+        <v>35.42426152165933</v>
       </c>
       <c r="D19" s="19" t="n">
-        <v>1845.735003003669</v>
+        <v>1680.322562782809</v>
       </c>
       <c r="E19" s="20">
         <f>MIN(C19,$B$3)*D19</f>
@@ -2427,7 +2427,7 @@
         <v/>
       </c>
       <c r="I19" s="21" t="n">
-        <v>12024.10549774539</v>
+        <v>28196.34138802607</v>
       </c>
       <c r="J19" s="20">
         <f>MIN(I19,H19)</f>
@@ -2450,17 +2450,17 @@
     <row r="20">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>0bc8522b-2de5-402b-b82e-ebb534151ee9</t>
+          <t>002e15d9-b27f-4a99-b94d-703b11215eab</t>
         </is>
       </c>
       <c r="B20" s="17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C20" s="18" t="n">
-        <v>336.6041633096748</v>
+        <v>250.3366353397119</v>
       </c>
       <c r="D20" s="19" t="n">
-        <v>1750.105740634113</v>
+        <v>628.0497454063474</v>
       </c>
       <c r="E20" s="20">
         <f>MIN(C20,$B$3)*D20</f>
@@ -2478,7 +2478,7 @@
         <v/>
       </c>
       <c r="I20" s="21" t="n">
-        <v>25486.87947007395</v>
+        <v>110595.9448259745</v>
       </c>
       <c r="J20" s="20">
         <f>MIN(I20,H20)</f>
@@ -2501,17 +2501,17 @@
     <row r="21">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>0fb3766f-33f4-4b9d-95c4-74dbfc6876dd</t>
+          <t>003d3c1a-1508-4af9-9994-80fcb20c6db5</t>
         </is>
       </c>
       <c r="B21" s="17" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C21" s="18" t="n">
-        <v>34.1265011384118</v>
+        <v>22.79816899118379</v>
       </c>
       <c r="D21" s="19" t="n">
-        <v>2173.314579577944</v>
+        <v>1224.825934646096</v>
       </c>
       <c r="E21" s="20">
         <f>MIN(C21,$B$3)*D21</f>
@@ -2529,7 +2529,7 @@
         <v/>
       </c>
       <c r="I21" s="21" t="n">
-        <v>31211.92177826306</v>
+        <v>25255.69997299017</v>
       </c>
       <c r="J21" s="20">
         <f>MIN(I21,H21)</f>
@@ -2552,24 +2552,24 @@
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t>0035a155-c4d3-4860-80e0-6c17481b3d61</t>
+          <t>007dffa2-4fe6-481f-8915-03b58be4847f</t>
         </is>
       </c>
       <c r="B22" s="17" t="n">
-        <v>1</v>
+        <v>78</v>
       </c>
       <c r="C22" s="18" t="n">
-        <v>0</v>
+        <v>425.7553115921269</v>
       </c>
       <c r="D22" s="19" t="n">
-        <v>1125.800303002638</v>
+        <v>2190.43015661056</v>
       </c>
       <c r="E22" s="20">
         <f>MIN(C22,$B$3)*D22</f>
         <v/>
       </c>
       <c r="F22" s="21" t="n">
-        <v>6586.879167817168</v>
+        <v>546195.6367360938</v>
       </c>
       <c r="G22" s="20">
         <f>MIN(F22,$B$4*B22)</f>
@@ -2580,7 +2580,7 @@
         <v/>
       </c>
       <c r="I22" s="21" t="n">
-        <v>13769.2550013806</v>
+        <v>758079.085775261</v>
       </c>
       <c r="J22" s="20">
         <f>MIN(I22,H22)</f>
@@ -2603,24 +2603,24 @@
     <row r="23">
       <c r="A23" s="16" t="inlineStr">
         <is>
-          <t>00745333-cf86-4178-8cf6-cd6f9d7d5cbd</t>
+          <t>00a83d76-9c9c-4d92-8d56-b16f1336cabb</t>
         </is>
       </c>
       <c r="B23" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C23" s="18" t="n">
-        <v>0</v>
+        <v>167.0618194984942</v>
       </c>
       <c r="D23" s="19" t="n">
-        <v>990.5549772618464</v>
+        <v>813.7362107148437</v>
       </c>
       <c r="E23" s="20">
         <f>MIN(C23,$B$3)*D23</f>
         <v/>
       </c>
       <c r="F23" s="21" t="n">
-        <v>13056.42456706143</v>
+        <v>33453.62511700418</v>
       </c>
       <c r="G23" s="20">
         <f>MIN(F23,$B$4*B23)</f>
@@ -2631,7 +2631,7 @@
         <v/>
       </c>
       <c r="I23" s="21" t="n">
-        <v>22609.3449544974</v>
+        <v>102502.5713358697</v>
       </c>
       <c r="J23" s="20">
         <f>MIN(I23,H23)</f>
@@ -2654,24 +2654,24 @@
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
         <is>
-          <t>00a83d76-9c9c-4d92-8d56-b16f1336cabb</t>
+          <t>00b30852-560a-437d-80fa-4ea99252c9bd</t>
         </is>
       </c>
       <c r="B24" s="17" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="18" t="n">
-        <v>0</v>
+        <v>98.61312973755619</v>
       </c>
       <c r="D24" s="19" t="n">
-        <v>909.0124673749219</v>
+        <v>1034.92968947975</v>
       </c>
       <c r="E24" s="20">
         <f>MIN(C24,$B$3)*D24</f>
         <v/>
       </c>
       <c r="F24" s="21" t="n">
-        <v>14543.84334445007</v>
+        <v>28945.23523399428</v>
       </c>
       <c r="G24" s="20">
         <f>MIN(F24,$B$4*B24)</f>
@@ -2682,7 +2682,7 @@
         <v/>
       </c>
       <c r="I24" s="21" t="n">
-        <v>25649.37321467409</v>
+        <v>95247.96177600817</v>
       </c>
       <c r="J24" s="20">
         <f>MIN(I24,H24)</f>
@@ -2705,24 +2705,24 @@
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
         <is>
-          <t>01b4d137-3ac2-408b-9de3-c572fc374ef4</t>
+          <t>00ffe249-5edc-4469-92f3-ff5339ea7ebf</t>
         </is>
       </c>
       <c r="B25" s="17" t="n">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="C25" s="18" t="n">
-        <v>472.2458906978015</v>
+        <v>94.3716013221896</v>
       </c>
       <c r="D25" s="19" t="n">
-        <v>1669.724652985133</v>
+        <v>2683.933480979382</v>
       </c>
       <c r="E25" s="20">
         <f>MIN(C25,$B$3)*D25</f>
         <v/>
       </c>
       <c r="F25" s="21" t="n">
-        <v>16284.16555913016</v>
+        <v>41807.03004206949</v>
       </c>
       <c r="G25" s="20">
         <f>MIN(F25,$B$4*B25)</f>
@@ -2733,7 +2733,7 @@
         <v/>
       </c>
       <c r="I25" s="21" t="n">
-        <v>27251.29860450401</v>
+        <v>72084.62540696503</v>
       </c>
       <c r="J25" s="20">
         <f>MIN(I25,H25)</f>
@@ -2763,10 +2763,10 @@
         <v>29</v>
       </c>
       <c r="C26" s="18" t="n">
-        <v>2824.033182987902</v>
+        <v>2750.306117999842</v>
       </c>
       <c r="D26" s="19" t="n">
-        <v>1908.027810002991</v>
+        <v>997.2180174243152</v>
       </c>
       <c r="E26" s="20">
         <f>MIN(C26,$B$3)*D26</f>
@@ -2814,10 +2814,10 @@
         <v>1</v>
       </c>
       <c r="C27" s="18" t="n">
-        <v>286.0372101473818</v>
+        <v>161.9731377315255</v>
       </c>
       <c r="D27" s="19" t="n">
-        <v>1891.519728815266</v>
+        <v>2740.833301343127</v>
       </c>
       <c r="E27" s="20">
         <f>MIN(C27,$B$3)*D27</f>
@@ -2858,17 +2858,17 @@
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t>001e2f9c-9846-4a4d-aff2-1de9e7b091c7</t>
+          <t>0055aa62-333d-49e8-8a1b-4277448835ed</t>
         </is>
       </c>
       <c r="B28" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="C28" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="C28" s="18" t="n">
-        <v>192.3987560767283</v>
-      </c>
       <c r="D28" s="19" t="n">
-        <v>1603.475556633135</v>
+        <v>2715.554313807805</v>
       </c>
       <c r="E28" s="20">
         <f>MIN(C28,$B$3)*D28</f>
@@ -2886,7 +2886,7 @@
         <v/>
       </c>
       <c r="I28" s="21" t="n">
-        <v>1725</v>
+        <v>575</v>
       </c>
       <c r="J28" s="20">
         <f>MIN(I28,H28)</f>
@@ -2909,17 +2909,17 @@
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
         <is>
-          <t>0055aa62-333d-49e8-8a1b-4277448835ed</t>
+          <t>00745333-cf86-4178-8cf6-cd6f9d7d5cbd</t>
         </is>
       </c>
       <c r="B29" s="17" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C29" s="18" t="n">
-        <v>212.7684182341731</v>
+        <v>0</v>
       </c>
       <c r="D29" s="19" t="n">
-        <v>1832.043468426193</v>
+        <v>1253.592714592957</v>
       </c>
       <c r="E29" s="20">
         <f>MIN(C29,$B$3)*D29</f>
@@ -2937,7 +2937,7 @@
         <v/>
       </c>
       <c r="I29" s="21" t="n">
-        <v>575</v>
+        <v>0</v>
       </c>
       <c r="J29" s="20">
         <f>MIN(I29,H29)</f>
@@ -2953,24 +2953,24 @@
       </c>
       <c r="M29" s="22" t="inlineStr">
         <is>
-          <t>liquefaction only</t>
+          <t>several dwellings</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="16" t="inlineStr">
         <is>
-          <t>002e15d9-b27f-4a99-b94d-703b11215eab</t>
+          <t>0078e0fc-2637-4256-9eb7-fbcc31d32e82</t>
         </is>
       </c>
       <c r="B30" s="17" t="n">
-        <v>3</v>
+        <v>204</v>
       </c>
       <c r="C30" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D30" s="19" t="n">
-        <v>816.216729440072</v>
+        <v>2252.313011387968</v>
       </c>
       <c r="E30" s="20">
         <f>MIN(C30,$B$3)*D30</f>
@@ -2988,7 +2988,7 @@
         <v/>
       </c>
       <c r="I30" s="21" t="n">
-        <v>0</v>
+        <v>575</v>
       </c>
       <c r="J30" s="20">
         <f>MIN(I30,H30)</f>
@@ -3004,24 +3004,24 @@
       </c>
       <c r="M30" s="22" t="inlineStr">
         <is>
-          <t>several dwellings</t>
+          <t>paid nothing, excess took it</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="16" t="inlineStr">
         <is>
-          <t>0078e0fc-2637-4256-9eb7-fbcc31d32e82</t>
+          <t>0120d782-7901-4838-9ae8-012ec8626771</t>
         </is>
       </c>
       <c r="B31" s="17" t="n">
-        <v>204</v>
+        <v>2</v>
       </c>
       <c r="C31" s="18" t="n">
-        <v>9455.37551407438</v>
+        <v>0</v>
       </c>
       <c r="D31" s="19" t="n">
-        <v>1914.25567961288</v>
+        <v>1951.33667089501</v>
       </c>
       <c r="E31" s="20">
         <f>MIN(C31,$B$3)*D31</f>
@@ -3039,7 +3039,7 @@
         <v/>
       </c>
       <c r="I31" s="21" t="n">
-        <v>1725</v>
+        <v>230</v>
       </c>
       <c r="J31" s="20">
         <f>MIN(I31,H31)</f>
@@ -3062,17 +3062,17 @@
     <row r="32">
       <c r="A32" s="16" t="inlineStr">
         <is>
-          <t>00ac4d7e-2245-4bfa-b36a-ef65994b6d02</t>
+          <t>0035a155-c4d3-4860-80e0-6c17481b3d61</t>
         </is>
       </c>
       <c r="B32" s="17" t="n">
-        <v>80</v>
+        <v>1</v>
       </c>
       <c r="C32" s="18" t="n">
-        <v>2098.301874066376</v>
+        <v>0</v>
       </c>
       <c r="D32" s="19" t="n">
-        <v>1603.806741137101</v>
+        <v>2100.83789056557</v>
       </c>
       <c r="E32" s="20">
         <f>MIN(C32,$B$3)*D32</f>
@@ -3090,7 +3090,7 @@
         <v/>
       </c>
       <c r="I32" s="21" t="n">
-        <v>1725</v>
+        <v>0</v>
       </c>
       <c r="J32" s="20">
         <f>MIN(I32,H32)</f>
@@ -3106,24 +3106,24 @@
       </c>
       <c r="M32" s="22" t="inlineStr">
         <is>
-          <t>paid nothing, excess took it</t>
+          <t>ordinary claim</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
         <is>
-          <t>00224faa-3597-401e-b493-559fc185861b</t>
+          <t>0056ff07-ee70-495f-9a55-26d6aed9bd34</t>
         </is>
       </c>
       <c r="B33" s="17" t="n">
         <v>1</v>
       </c>
       <c r="C33" s="18" t="n">
-        <v>0</v>
+        <v>28.28705013766703</v>
       </c>
       <c r="D33" s="19" t="n">
-        <v>1142.349530467185</v>
+        <v>1348.528388619784</v>
       </c>
       <c r="E33" s="20">
         <f>MIN(C33,$B$3)*D33</f>
@@ -3141,7 +3141,7 @@
         <v/>
       </c>
       <c r="I33" s="21" t="n">
-        <v>0</v>
+        <v>32300.13781586216</v>
       </c>
       <c r="J33" s="20">
         <f>MIN(I33,H33)</f>
@@ -3530,41 +3530,45 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>03dc0301-b79a-4927-9dc7-cd7e95fc9aaf</t>
+          <t>018d3ae8-debe-4c14-8b06-2870c121761e</t>
         </is>
       </c>
       <c r="B6" s="28" t="n">
-        <v>0</v>
+        <v>0.9297514124773443</v>
       </c>
       <c r="C6" s="28" t="n">
-        <v>3.994276433826656</v>
+        <v>0</v>
       </c>
       <c r="D6" s="28" t="n"/>
       <c r="E6" s="28" t="n">
-        <v>3.994276433826656</v>
+        <v>0.9297514124773443</v>
       </c>
       <c r="F6" s="29" t="n">
-        <v>906.9153731669335</v>
+        <v>1643.133438311629</v>
       </c>
       <c r="G6" s="30">
         <f>MIN(E6,Calculation!$B$3)*F6</f>
         <v/>
       </c>
-      <c r="H6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>small</t>
+        </is>
+      </c>
       <c r="I6" s="31" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="J6" s="28" t="n">
-        <v>0</v>
+        <v>5.363635884301483</v>
       </c>
       <c r="K6" s="32" t="n">
-        <v>0</v>
+        <v>3104.853267981484</v>
       </c>
       <c r="L6" s="28" t="n">
-        <v>1.884367009081398</v>
+        <v>0</v>
       </c>
       <c r="M6" s="32" t="n">
-        <v>282.6550513622097</v>
+        <v>0</v>
       </c>
       <c r="N6" s="30">
         <f>K6+M6</f>
@@ -3572,43 +3576,39 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>shaking</t>
+          <t>no wall on the property</t>
         </is>
       </c>
       <c r="P6" s="4" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>none</t>
         </is>
       </c>
       <c r="Q6" s="31" t="n">
-        <v>1.75</v>
+        <v>0</v>
       </c>
       <c r="R6" s="28" t="n">
-        <v>6.313108289984361</v>
+        <v>0</v>
       </c>
       <c r="S6" s="29" t="n">
-        <v>744.6900000000001</v>
+        <v>0</v>
       </c>
       <c r="T6" s="32" t="n">
-        <v>8227.290071819794</v>
+        <v>0</v>
       </c>
       <c r="U6" s="30">
         <f>T6*(1+Calculation!$B$7)</f>
         <v/>
       </c>
-      <c r="V6" s="4" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
+      <c r="V6" s="4" t="inlineStr"/>
       <c r="W6" s="28" t="n">
-        <v>6.826402814117852</v>
+        <v>0</v>
       </c>
       <c r="X6" s="29" t="n">
-        <v>744.6900000000002</v>
+        <v>0</v>
       </c>
       <c r="Y6" s="32" t="n">
-        <v>11209.23637517816</v>
+        <v>0</v>
       </c>
       <c r="Z6" s="28" t="n"/>
       <c r="AA6" s="28" t="n"/>
@@ -3616,7 +3616,7 @@
         <v>0</v>
       </c>
       <c r="AC6" s="28" t="n">
-        <v>159.4213451242771</v>
+        <v>245.0598163514067</v>
       </c>
       <c r="AD6" s="33" t="n">
         <v>0</v>
@@ -3632,7 +3632,7 @@
         <v>1</v>
       </c>
       <c r="AH6" s="32" t="n">
-        <v>5355</v>
+        <v>5100</v>
       </c>
       <c r="AI6" s="30">
         <f>N6+Y6+AF6+AH6</f>
@@ -3681,21 +3681,21 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>331011f8-ce50-46ad-9aeb-03fffa6c8506</t>
+          <t>01f4c88f-c20c-48a2-a1e1-c3994510daa1</t>
         </is>
       </c>
       <c r="B7" s="28" t="n">
-        <v>11.61980777911261</v>
+        <v>0.6900666733749836</v>
       </c>
       <c r="C7" s="28" t="n">
-        <v>0</v>
+        <v>0.9524061830173011</v>
       </c>
       <c r="D7" s="28" t="n"/>
       <c r="E7" s="28" t="n">
-        <v>11.61980777911261</v>
+        <v>1.642472856392285</v>
       </c>
       <c r="F7" s="29" t="n">
-        <v>875.2256394431051</v>
+        <v>1610.224150599341</v>
       </c>
       <c r="G7" s="30">
         <f>MIN(E7,Calculation!$B$3)*F7</f>
@@ -3712,10 +3712,10 @@
         <v>0</v>
       </c>
       <c r="L7" s="28" t="n">
-        <v>0</v>
+        <v>0.7677247428549417</v>
       </c>
       <c r="M7" s="32" t="n">
-        <v>0</v>
+        <v>115.1587114282413</v>
       </c>
       <c r="N7" s="30">
         <f>K7+M7</f>
@@ -3723,25 +3723,25 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>shaking + evacuated</t>
+          <t>evacuated</t>
         </is>
       </c>
       <c r="P7" s="4" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>small</t>
         </is>
       </c>
       <c r="Q7" s="31" t="n">
-        <v>2.75</v>
+        <v>0.75</v>
       </c>
       <c r="R7" s="28" t="n">
-        <v>8.159218973584622</v>
+        <v>4.658655447551695</v>
       </c>
       <c r="S7" s="29" t="n">
-        <v>798.8</v>
+        <v>643.1900000000001</v>
       </c>
       <c r="T7" s="32" t="n">
-        <v>17923.35631927334</v>
+        <v>2247.300447983081</v>
       </c>
       <c r="U7" s="30">
         <f>T7*(1+Calculation!$B$7)</f>
@@ -3749,17 +3749,17 @@
       </c>
       <c r="V7" s="4" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>small</t>
         </is>
       </c>
       <c r="W7" s="28" t="n">
-        <v>8.820748443781859</v>
+        <v>5.81244191983759</v>
       </c>
       <c r="X7" s="29" t="n">
-        <v>798.8000000000001</v>
+        <v>643.1900000000001</v>
       </c>
       <c r="Y7" s="32" t="n">
-        <v>26739.62258690874</v>
+        <v>3532.886769907221</v>
       </c>
       <c r="Z7" s="28" t="n"/>
       <c r="AA7" s="28" t="n"/>
@@ -3767,7 +3767,7 @@
         <v>0</v>
       </c>
       <c r="AC7" s="28" t="n">
-        <v>266.2914170356131</v>
+        <v>183.015131107938</v>
       </c>
       <c r="AD7" s="33" t="n">
         <v>0</v>
@@ -3783,7 +3783,7 @@
         <v>1</v>
       </c>
       <c r="AH7" s="32" t="n">
-        <v>5865</v>
+        <v>5355</v>
       </c>
       <c r="AI7" s="30">
         <f>N7+Y7+AF7+AH7</f>
@@ -3832,21 +3832,21 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>36df7f1f-d454-4fd8-9751-1db3ad4e883a</t>
+          <t>01f97a58-c26c-468a-b02f-b75858b5575b</t>
         </is>
       </c>
       <c r="B8" s="28" t="n">
-        <v>2.739921778496873</v>
+        <v>9.544239917306806</v>
       </c>
       <c r="C8" s="28" t="n">
-        <v>5.254910674327312</v>
+        <v>1.339097901247442</v>
       </c>
       <c r="D8" s="28" t="n"/>
       <c r="E8" s="28" t="n">
-        <v>5.254910674327313</v>
+        <v>10.88333781855425</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>1033.806982141251</v>
+        <v>1991.793188542959</v>
       </c>
       <c r="G8" s="30">
         <f>MIN(E8,Calculation!$B$3)*F8</f>
@@ -3854,23 +3854,23 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I8" s="31" t="n">
-        <v>0.75</v>
+        <v>1.75</v>
       </c>
       <c r="J8" s="28" t="n">
-        <v>7.241885461988845</v>
+        <v>8.665476999954935</v>
       </c>
       <c r="K8" s="32" t="n">
-        <v>4611.329227193641</v>
+        <v>14229.07241794765</v>
       </c>
       <c r="L8" s="28" t="n">
-        <v>2.364807321606506</v>
+        <v>0.8266304144196229</v>
       </c>
       <c r="M8" s="32" t="n">
-        <v>354.7210982409759</v>
+        <v>123.9945621629434</v>
       </c>
       <c r="N8" s="30">
         <f>K8+M8</f>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>wall present, undamaged</t>
+          <t>no wall on the property</t>
         </is>
       </c>
       <c r="P8" s="4" t="inlineStr">
@@ -3918,7 +3918,7 @@
         <v>0</v>
       </c>
       <c r="AC8" s="28" t="n">
-        <v>420.2371467194171</v>
+        <v>144.9001795627513</v>
       </c>
       <c r="AD8" s="33" t="n">
         <v>0</v>
@@ -3931,10 +3931,10 @@
         <v>0</v>
       </c>
       <c r="AG8" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH8" s="32" t="n">
-        <v>5610</v>
+        <v>5355</v>
       </c>
       <c r="AI8" s="30">
         <f>N8+Y8+AF8+AH8</f>
@@ -3983,21 +3983,21 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>3c9cb87a-ae7d-4616-b2f0-ffff94a2930b</t>
+          <t>02d672fd-0ee8-4e6a-9e86-e092694dc40f</t>
         </is>
       </c>
       <c r="B9" s="28" t="n">
-        <v>4.81379863873295</v>
+        <v>0</v>
       </c>
       <c r="C9" s="28" t="n">
-        <v>83.99693044062863</v>
+        <v>0.291589490021579</v>
       </c>
       <c r="D9" s="28" t="n"/>
       <c r="E9" s="28" t="n">
-        <v>83.99693044062862</v>
+        <v>0.291589490021579</v>
       </c>
       <c r="F9" s="29" t="n">
-        <v>952.5188914254333</v>
+        <v>2002.415796489682</v>
       </c>
       <c r="G9" s="30">
         <f>MIN(E9,Calculation!$B$3)*F9</f>
@@ -4005,23 +4005,23 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>small</t>
         </is>
       </c>
       <c r="I9" s="31" t="n">
-        <v>2.75</v>
+        <v>0.75</v>
       </c>
       <c r="J9" s="28" t="n">
-        <v>16.96124457300522</v>
+        <v>5</v>
       </c>
       <c r="K9" s="32" t="n">
-        <v>51417.09701585837</v>
+        <v>2894.355</v>
       </c>
       <c r="L9" s="28" t="n">
-        <v>100.6916108565515</v>
+        <v>0.2664067134254555</v>
       </c>
       <c r="M9" s="32" t="n">
-        <v>15103.74162848273</v>
+        <v>39.96100701381833</v>
       </c>
       <c r="N9" s="30">
         <f>K9+M9</f>
@@ -4066,26 +4066,26 @@
       <c r="Z9" s="28" t="n"/>
       <c r="AA9" s="28" t="n"/>
       <c r="AB9" s="28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC9" s="28" t="n">
-        <v>447.623704376365</v>
+        <v>249.6514398579299</v>
       </c>
       <c r="AD9" s="33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE9" s="30">
         <f>MIN(AB9,Calculation!$B$3)*F9</f>
         <v/>
       </c>
       <c r="AF9" s="32" t="n">
-        <v>0</v>
+        <v>500.0000000000001</v>
       </c>
       <c r="AG9" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH9" s="32" t="n">
-        <v>5865</v>
+        <v>5100</v>
       </c>
       <c r="AI9" s="30">
         <f>N9+Y9+AF9+AH9</f>
@@ -4134,21 +4134,21 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>06953c1e-a185-4880-a3e8-203ab7d4220a</t>
+          <t>001e2f9c-9846-4a4d-aff2-1de9e7b091c7</t>
         </is>
       </c>
       <c r="B10" s="28" t="n">
-        <v>25.76580155440493</v>
+        <v>10.18827772606164</v>
       </c>
       <c r="C10" s="28" t="n">
-        <v>23.23198887690671</v>
+        <v>2</v>
       </c>
       <c r="D10" s="28" t="n"/>
       <c r="E10" s="28" t="n">
-        <v>31.56185795826037</v>
+        <v>12.18827772606164</v>
       </c>
       <c r="F10" s="29" t="n">
-        <v>1215.255114101618</v>
+        <v>2915.070027166179</v>
       </c>
       <c r="G10" s="30">
         <f>MIN(E10,Calculation!$B$3)*F10</f>
@@ -4163,16 +4163,16 @@
         <v>1.75</v>
       </c>
       <c r="J10" s="28" t="n">
-        <v>11.94504348109692</v>
+        <v>8.937261938779761</v>
       </c>
       <c r="K10" s="32" t="n">
-        <v>22416.29316344393</v>
+        <v>13976.52814569879</v>
       </c>
       <c r="L10" s="28" t="n">
-        <v>7.050430954134018</v>
+        <v>3.087421228017586</v>
       </c>
       <c r="M10" s="32" t="n">
-        <v>1057.564643120103</v>
+        <v>463.1131842026378</v>
       </c>
       <c r="N10" s="30">
         <f>K10+M10</f>
@@ -4217,26 +4217,26 @@
       <c r="Z10" s="28" t="n"/>
       <c r="AA10" s="28" t="n"/>
       <c r="AB10" s="28" t="n">
-        <v>0</v>
+        <v>75.53717854302793</v>
       </c>
       <c r="AC10" s="28" t="n">
-        <v>50447.22716690691</v>
+        <v>192.3987560767283</v>
       </c>
       <c r="AD10" s="33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AE10" s="30">
         <f>MIN(AB10,Calculation!$B$3)*F10</f>
         <v/>
       </c>
       <c r="AF10" s="32" t="n">
-        <v>200</v>
+        <v>1500</v>
       </c>
       <c r="AG10" s="34" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AH10" s="32" t="n">
-        <v>6120</v>
+        <v>5100</v>
       </c>
       <c r="AI10" s="30">
         <f>N10+Y10+AF10+AH10</f>
@@ -4285,21 +4285,21 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>0af1f540-21f2-4654-97ed-047e9a0d7e42</t>
+          <t>00224faa-3597-401e-b493-559fc185861b</t>
         </is>
       </c>
       <c r="B11" s="28" t="n">
-        <v>5.636895421053411</v>
+        <v>35.42426152165933</v>
       </c>
       <c r="C11" s="28" t="n">
-        <v>3.183434007476635</v>
+        <v>0</v>
       </c>
       <c r="D11" s="28" t="n"/>
       <c r="E11" s="28" t="n">
-        <v>5.903114465110614</v>
+        <v>35.42426152165933</v>
       </c>
       <c r="F11" s="29" t="n">
-        <v>1845.735003003669</v>
+        <v>1680.322562782809</v>
       </c>
       <c r="G11" s="30">
         <f>MIN(E11,Calculation!$B$3)*F11</f>
@@ -4307,23 +4307,23 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I11" s="31" t="n">
-        <v>0.75</v>
+        <v>1.75</v>
       </c>
       <c r="J11" s="28" t="n">
-        <v>7.436019343691363</v>
+        <v>12.41715647016964</v>
       </c>
       <c r="K11" s="32" t="n">
-        <v>4519.720751177061</v>
+        <v>19418.55772871832</v>
       </c>
       <c r="L11" s="28" t="n">
-        <v>0.5401543993725951</v>
+        <v>0</v>
       </c>
       <c r="M11" s="32" t="n">
-        <v>81.02315990588927</v>
+        <v>0</v>
       </c>
       <c r="N11" s="30">
         <f>K11+M11</f>
@@ -4368,26 +4368,26 @@
       <c r="Z11" s="28" t="n"/>
       <c r="AA11" s="28" t="n"/>
       <c r="AB11" s="28" t="n">
-        <v>356.3788137462104</v>
+        <v>0</v>
       </c>
       <c r="AC11" s="28" t="n">
-        <v>356.3788137462104</v>
+        <v>394.0728141999576</v>
       </c>
       <c r="AD11" s="33" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AE11" s="30">
         <f>MIN(AB11,Calculation!$B$3)*F11</f>
         <v/>
       </c>
       <c r="AF11" s="32" t="n">
-        <v>500.0000000000001</v>
+        <v>0</v>
       </c>
       <c r="AG11" s="34" t="n">
         <v>1</v>
       </c>
       <c r="AH11" s="32" t="n">
-        <v>5355</v>
+        <v>5100</v>
       </c>
       <c r="AI11" s="30">
         <f>N11+Y11+AF11+AH11</f>
@@ -4436,21 +4436,21 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>0bc8522b-2de5-402b-b82e-ebb534151ee9</t>
+          <t>002e15d9-b27f-4a99-b94d-703b11215eab</t>
         </is>
       </c>
       <c r="B12" s="28" t="n">
-        <v>15.48983220842302</v>
+        <v>83.34188390833913</v>
       </c>
       <c r="C12" s="28" t="n">
-        <v>8.547847131838395</v>
+        <v>240.4011895337888</v>
       </c>
       <c r="D12" s="28" t="n"/>
       <c r="E12" s="28" t="n">
-        <v>15.48983220842302</v>
+        <v>250.3366353397119</v>
       </c>
       <c r="F12" s="29" t="n">
-        <v>1750.105740634113</v>
+        <v>628.0497454063474</v>
       </c>
       <c r="G12" s="30">
         <f>MIN(E12,Calculation!$B$3)*F12</f>
@@ -4458,23 +4458,23 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="I12" s="31" t="n">
-        <v>1.75</v>
+        <v>2.75</v>
       </c>
       <c r="J12" s="28" t="n">
-        <v>9.565937873965719</v>
+        <v>26.37572950049727</v>
       </c>
       <c r="K12" s="32" t="n">
-        <v>14959.68237826341</v>
+        <v>79956.59969136443</v>
       </c>
       <c r="L12" s="28" t="n">
-        <v>4.018810058382776</v>
+        <v>68.99191409220519</v>
       </c>
       <c r="M12" s="32" t="n">
-        <v>602.8215087574164</v>
+        <v>10348.78711383078</v>
       </c>
       <c r="N12" s="30">
         <f>K12+M12</f>
@@ -4519,26 +4519,26 @@
       <c r="Z12" s="28" t="n"/>
       <c r="AA12" s="28" t="n"/>
       <c r="AB12" s="28" t="n">
-        <v>336.6041633096748</v>
+        <v>0</v>
       </c>
       <c r="AC12" s="28" t="n">
-        <v>336.6041633096748</v>
+        <v>252.3366353326147</v>
       </c>
       <c r="AD12" s="33" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AE12" s="30">
         <f>MIN(AB12,Calculation!$B$3)*F12</f>
         <v/>
       </c>
       <c r="AF12" s="32" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="AG12" s="34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AH12" s="32" t="n">
-        <v>5100</v>
+        <v>5865</v>
       </c>
       <c r="AI12" s="30">
         <f>N12+Y12+AF12+AH12</f>
@@ -4587,21 +4587,21 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>0fb3766f-33f4-4b9d-95c4-74dbfc6876dd</t>
+          <t>003d3c1a-1508-4af9-9994-80fcb20c6db5</t>
         </is>
       </c>
       <c r="B13" s="28" t="n">
-        <v>28.16598323933578</v>
+        <v>0.2802026608601492</v>
       </c>
       <c r="C13" s="28" t="n">
-        <v>28.16598323933578</v>
+        <v>22.51796633032364</v>
       </c>
       <c r="D13" s="28" t="n"/>
       <c r="E13" s="28" t="n">
-        <v>34.1265011384118</v>
+        <v>22.79816899118379</v>
       </c>
       <c r="F13" s="29" t="n">
-        <v>2173.314579577944</v>
+        <v>1224.825934646096</v>
       </c>
       <c r="G13" s="30">
         <f>MIN(E13,Calculation!$B$3)*F13</f>
@@ -4616,16 +4616,16 @@
         <v>1.75</v>
       </c>
       <c r="J13" s="28" t="n">
-        <v>12.26153752499035</v>
+        <v>10.75250605200525</v>
       </c>
       <c r="K13" s="32" t="n">
-        <v>20133.95285676456</v>
+        <v>16815.29583692236</v>
       </c>
       <c r="L13" s="28" t="n">
-        <v>9.678991263674343</v>
+        <v>0.3078826697360007</v>
       </c>
       <c r="M13" s="32" t="n">
-        <v>1451.848689551151</v>
+        <v>46.1824004604001</v>
       </c>
       <c r="N13" s="30">
         <f>K13+M13</f>
@@ -4673,23 +4673,23 @@
         <v>0</v>
       </c>
       <c r="AC13" s="28" t="n">
-        <v>836.0527260023529</v>
+        <v>287.5698235696805</v>
       </c>
       <c r="AD13" s="33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE13" s="30">
         <f>MIN(AB13,Calculation!$B$3)*F13</f>
         <v/>
       </c>
       <c r="AF13" s="32" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AG13" s="34" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AH13" s="32" t="n">
-        <v>5355</v>
+        <v>5100</v>
       </c>
       <c r="AI13" s="30">
         <f>N13+Y13+AF13+AH13</f>
@@ -4738,21 +4738,21 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>0035a155-c4d3-4860-80e0-6c17481b3d61</t>
+          <t>007dffa2-4fe6-481f-8915-03b58be4847f</t>
         </is>
       </c>
       <c r="B14" s="28" t="n">
-        <v>0</v>
+        <v>252.6370903825587</v>
       </c>
       <c r="C14" s="28" t="n">
-        <v>0</v>
+        <v>173.1182212095682</v>
       </c>
       <c r="D14" s="28" t="n"/>
       <c r="E14" s="28" t="n">
-        <v>0</v>
+        <v>425.7553115921269</v>
       </c>
       <c r="F14" s="29" t="n">
-        <v>1125.800303002638</v>
+        <v>2190.43015661056</v>
       </c>
       <c r="G14" s="30">
         <f>MIN(E14,Calculation!$B$3)*F14</f>
@@ -4769,10 +4769,10 @@
         <v>0</v>
       </c>
       <c r="L14" s="28" t="n">
-        <v>0</v>
+        <v>177.6773639629978</v>
       </c>
       <c r="M14" s="32" t="n">
-        <v>0</v>
+        <v>26651.60459444967</v>
       </c>
       <c r="N14" s="30">
         <f>K14+M14</f>
@@ -4780,25 +4780,25 @@
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>shaking</t>
+          <t>shaking + evacuated, shaking + evacuated + inundated</t>
         </is>
       </c>
       <c r="P14" s="4" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>large</t>
         </is>
       </c>
       <c r="Q14" s="31" t="n">
-        <v>0.75</v>
+        <v>2.75</v>
       </c>
       <c r="R14" s="28" t="n">
-        <v>6.238939737591432</v>
+        <v>218.8214568128634</v>
       </c>
       <c r="S14" s="29" t="n">
         <v>1224.08</v>
       </c>
       <c r="T14" s="32" t="n">
-        <v>5727.72101549319</v>
+        <v>474952.7275966033</v>
       </c>
       <c r="U14" s="30">
         <f>T14*(1+Calculation!$B$7)</f>
@@ -4806,17 +4806,17 @@
       </c>
       <c r="V14" s="4" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>large</t>
         </is>
       </c>
       <c r="W14" s="28" t="n">
-        <v>6.238939737591432</v>
+        <v>218.8214568128634</v>
       </c>
       <c r="X14" s="29" t="n">
-        <v>1224.08</v>
+        <v>932.8405814363465</v>
       </c>
       <c r="Y14" s="32" t="n">
-        <v>6873.265218591828</v>
+        <v>626937.6004275165</v>
       </c>
       <c r="Z14" s="28" t="n"/>
       <c r="AA14" s="28" t="n"/>
@@ -4824,7 +4824,7 @@
         <v>0</v>
       </c>
       <c r="AC14" s="28" t="n">
-        <v>155.6974761971898</v>
+        <v>7333.538575907865</v>
       </c>
       <c r="AD14" s="33" t="n">
         <v>0</v>
@@ -4837,10 +4837,10 @@
         <v>0</v>
       </c>
       <c r="AG14" s="34" t="n">
-        <v>1</v>
+        <v>78</v>
       </c>
       <c r="AH14" s="32" t="n">
-        <v>5100</v>
+        <v>5610</v>
       </c>
       <c r="AI14" s="30">
         <f>N14+Y14+AF14+AH14</f>
@@ -4889,21 +4889,21 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>00745333-cf86-4178-8cf6-cd6f9d7d5cbd</t>
+          <t>00a83d76-9c9c-4d92-8d56-b16f1336cabb</t>
         </is>
       </c>
       <c r="B15" s="28" t="n">
-        <v>0</v>
+        <v>67.57112205483558</v>
       </c>
       <c r="C15" s="28" t="n">
-        <v>0</v>
+        <v>117.6161420986407</v>
       </c>
       <c r="D15" s="28" t="n"/>
       <c r="E15" s="28" t="n">
-        <v>0</v>
+        <v>167.0618194984942</v>
       </c>
       <c r="F15" s="29" t="n">
-        <v>990.5549772618464</v>
+        <v>813.7362107148437</v>
       </c>
       <c r="G15" s="30">
         <f>MIN(E15,Calculation!$B$3)*F15</f>
@@ -4920,10 +4920,10 @@
         <v>0</v>
       </c>
       <c r="L15" s="28" t="n">
-        <v>0</v>
+        <v>104.8662413356522</v>
       </c>
       <c r="M15" s="32" t="n">
-        <v>0</v>
+        <v>15729.93620034783</v>
       </c>
       <c r="N15" s="30">
         <f>K15+M15</f>
@@ -4931,25 +4931,25 @@
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>shaking</t>
+          <t>shaking + evacuated + inundated</t>
         </is>
       </c>
       <c r="P15" s="4" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="Q15" s="31" t="n">
-        <v>1.75</v>
+        <v>2.75</v>
       </c>
       <c r="R15" s="28" t="n">
-        <v>8.711899422777982</v>
+        <v>13.24264068711929</v>
       </c>
       <c r="S15" s="29" t="n">
-        <v>744.6900000000001</v>
+        <v>798.8</v>
       </c>
       <c r="T15" s="32" t="n">
-        <v>11353.41266700994</v>
+        <v>29090.10879739494</v>
       </c>
       <c r="U15" s="30">
         <f>T15*(1+Calculation!$B$7)</f>
@@ -4957,17 +4957,17 @@
       </c>
       <c r="V15" s="4" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="W15" s="28" t="n">
-        <v>8.711899422777982</v>
+        <v>22.27904918197301</v>
       </c>
       <c r="X15" s="29" t="n">
-        <v>744.6900000000001</v>
+        <v>798.8</v>
       </c>
       <c r="Y15" s="32" t="n">
-        <v>14305.29996043252</v>
+        <v>67537.73452649536</v>
       </c>
       <c r="Z15" s="28" t="n"/>
       <c r="AA15" s="28" t="n"/>
@@ -4975,7 +4975,7 @@
         <v>0</v>
       </c>
       <c r="AC15" s="28" t="n">
-        <v>303.5887662103974</v>
+        <v>376.6999349914819</v>
       </c>
       <c r="AD15" s="33" t="n">
         <v>0</v>
@@ -4988,10 +4988,10 @@
         <v>0</v>
       </c>
       <c r="AG15" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH15" s="32" t="n">
-        <v>5355</v>
+        <v>5865</v>
       </c>
       <c r="AI15" s="30">
         <f>N15+Y15+AF15+AH15</f>
@@ -5040,21 +5040,21 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>00a83d76-9c9c-4d92-8d56-b16f1336cabb</t>
+          <t>00b30852-560a-437d-80fa-4ea99252c9bd</t>
         </is>
       </c>
       <c r="B16" s="28" t="n">
-        <v>0</v>
+        <v>66.67370675629941</v>
       </c>
       <c r="C16" s="28" t="n">
-        <v>0</v>
+        <v>31.93942298125679</v>
       </c>
       <c r="D16" s="28" t="n"/>
       <c r="E16" s="28" t="n">
-        <v>0</v>
+        <v>98.61312973755619</v>
       </c>
       <c r="F16" s="29" t="n">
-        <v>909.0124673749219</v>
+        <v>1034.92968947975</v>
       </c>
       <c r="G16" s="30">
         <f>MIN(E16,Calculation!$B$3)*F16</f>
@@ -5071,10 +5071,10 @@
         <v>0</v>
       </c>
       <c r="L16" s="28" t="n">
-        <v>0</v>
+        <v>59.96284602958234</v>
       </c>
       <c r="M16" s="32" t="n">
-        <v>0</v>
+        <v>8994.426904437352</v>
       </c>
       <c r="N16" s="30">
         <f>K16+M16</f>
@@ -5082,7 +5082,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>shaking</t>
+          <t>shaking + evacuated</t>
         </is>
       </c>
       <c r="P16" s="4" t="inlineStr">
@@ -5094,13 +5094,13 @@
         <v>1.75</v>
       </c>
       <c r="R16" s="28" t="n">
-        <v>9.70437961684674</v>
+        <v>19.31370849898476</v>
       </c>
       <c r="S16" s="29" t="n">
         <v>744.6900000000001</v>
       </c>
       <c r="T16" s="32" t="n">
-        <v>12646.8202995218</v>
+        <v>25169.76976869068</v>
       </c>
       <c r="U16" s="30">
         <f>T16*(1+Calculation!$B$7)</f>
@@ -5108,17 +5108,17 @@
       </c>
       <c r="V16" s="4" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="W16" s="28" t="n">
-        <v>9.70437961684674</v>
+        <v>27.286367381808</v>
       </c>
       <c r="X16" s="29" t="n">
-        <v>744.6900000000001</v>
+        <v>785.4979179620705</v>
       </c>
       <c r="Y16" s="32" t="n">
-        <v>16693.80279536877</v>
+        <v>68219.88768339585</v>
       </c>
       <c r="Z16" s="28" t="n"/>
       <c r="AA16" s="28" t="n"/>
@@ -5126,7 +5126,7 @@
         <v>0</v>
       </c>
       <c r="AC16" s="28" t="n">
-        <v>376.6999349914819</v>
+        <v>566.6526483765928</v>
       </c>
       <c r="AD16" s="33" t="n">
         <v>0</v>
@@ -5191,21 +5191,21 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>01b4d137-3ac2-408b-9de3-c572fc374ef4</t>
+          <t>00ffe249-5edc-4469-92f3-ff5339ea7ebf</t>
         </is>
       </c>
       <c r="B17" s="28" t="n">
-        <v>0</v>
+        <v>38.65951098903223</v>
       </c>
       <c r="C17" s="28" t="n">
-        <v>0</v>
+        <v>57.4775146358477</v>
       </c>
       <c r="D17" s="28" t="n"/>
       <c r="E17" s="28" t="n">
-        <v>0</v>
+        <v>94.3716013221896</v>
       </c>
       <c r="F17" s="29" t="n">
-        <v>1669.724652985133</v>
+        <v>2683.933480979382</v>
       </c>
       <c r="G17" s="30">
         <f>MIN(E17,Calculation!$B$3)*F17</f>
@@ -5222,10 +5222,10 @@
         <v>0</v>
       </c>
       <c r="L17" s="28" t="n">
-        <v>0</v>
+        <v>42.76525105680536</v>
       </c>
       <c r="M17" s="32" t="n">
-        <v>0</v>
+        <v>6414.787658520804</v>
       </c>
       <c r="N17" s="30">
         <f>K17+M17</f>
@@ -5233,7 +5233,7 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>shaking</t>
+          <t>shaking + evacuated + inundated</t>
         </is>
       </c>
       <c r="P17" s="4" t="inlineStr">
@@ -5245,13 +5245,13 @@
         <v>1.75</v>
       </c>
       <c r="R17" s="28" t="n">
-        <v>10.86560963197419</v>
+        <v>16.97085118947265</v>
       </c>
       <c r="S17" s="29" t="n">
-        <v>744.6900000000001</v>
+        <v>1224.08</v>
       </c>
       <c r="T17" s="32" t="n">
-        <v>14160.14396446101</v>
+        <v>36353.93916701695</v>
       </c>
       <c r="U17" s="30">
         <f>T17*(1+Calculation!$B$7)</f>
@@ -5263,21 +5263,21 @@
         </is>
       </c>
       <c r="W17" s="28" t="n">
-        <v>10.86560963197419</v>
+        <v>17.73838428070707</v>
       </c>
       <c r="X17" s="29" t="n">
-        <v>744.6900000000001</v>
+        <v>1224.08</v>
       </c>
       <c r="Y17" s="32" t="n">
-        <v>17841.78139522087</v>
+        <v>50157.49530405749</v>
       </c>
       <c r="Z17" s="28" t="n"/>
       <c r="AA17" s="28" t="n"/>
       <c r="AB17" s="28" t="n">
-        <v>472.2458906978015</v>
+        <v>1</v>
       </c>
       <c r="AC17" s="28" t="n">
-        <v>472.2458906978015</v>
+        <v>3311.143168208214</v>
       </c>
       <c r="AD17" s="33" t="n">
         <v>2</v>
@@ -5290,10 +5290,10 @@
         <v>500.0000000000001</v>
       </c>
       <c r="AG17" s="34" t="n">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="AH17" s="32" t="n">
-        <v>5355</v>
+        <v>5610</v>
       </c>
       <c r="AI17" s="30">
         <f>N17+Y17+AF17+AH17</f>
@@ -5356,7 +5356,7 @@
         <v>0</v>
       </c>
       <c r="F18" s="29" t="n">
-        <v>1908.027810002991</v>
+        <v>997.2180174243152</v>
       </c>
       <c r="G18" s="30">
         <f>MIN(E18,Calculation!$B$3)*F18</f>
@@ -5421,7 +5421,7 @@
       <c r="Z18" s="28" t="n"/>
       <c r="AA18" s="28" t="n"/>
       <c r="AB18" s="28" t="n">
-        <v>2824.033182987902</v>
+        <v>2750.306117999842</v>
       </c>
       <c r="AC18" s="28" t="n">
         <v>2824.033182987902</v>
@@ -5503,7 +5503,7 @@
         <v>0</v>
       </c>
       <c r="F19" s="29" t="n">
-        <v>1891.519728815266</v>
+        <v>2740.833301343127</v>
       </c>
       <c r="G19" s="30">
         <f>MIN(E19,Calculation!$B$3)*F19</f>
@@ -5568,7 +5568,7 @@
       <c r="Z19" s="28" t="n"/>
       <c r="AA19" s="28" t="n"/>
       <c r="AB19" s="28" t="n">
-        <v>286.0372101473818</v>
+        <v>161.9731377315255</v>
       </c>
       <c r="AC19" s="28" t="n">
         <v>286.0372101473818</v>
@@ -5636,7 +5636,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>001e2f9c-9846-4a4d-aff2-1de9e7b091c7</t>
+          <t>0055aa62-333d-49e8-8a1b-4277448835ed</t>
         </is>
       </c>
       <c r="B20" s="28" t="n">
@@ -5650,7 +5650,7 @@
         <v>0</v>
       </c>
       <c r="F20" s="29" t="n">
-        <v>1603.475556633135</v>
+        <v>2715.554313807805</v>
       </c>
       <c r="G20" s="30">
         <f>MIN(E20,Calculation!$B$3)*F20</f>
@@ -5715,23 +5715,23 @@
       <c r="Z20" s="28" t="n"/>
       <c r="AA20" s="28" t="n"/>
       <c r="AB20" s="28" t="n">
-        <v>192.3987560767283</v>
+        <v>1</v>
       </c>
       <c r="AC20" s="28" t="n">
-        <v>192.3987560767283</v>
+        <v>212.7684182341731</v>
       </c>
       <c r="AD20" s="33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AE20" s="30">
         <f>MIN(AB20,Calculation!$B$3)*F20</f>
         <v/>
       </c>
       <c r="AF20" s="32" t="n">
-        <v>1500</v>
+        <v>500.0000000000001</v>
       </c>
       <c r="AG20" s="34" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AH20" s="32" t="n">
         <v>0</v>
@@ -5783,7 +5783,7 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>0055aa62-333d-49e8-8a1b-4277448835ed</t>
+          <t>00745333-cf86-4178-8cf6-cd6f9d7d5cbd</t>
         </is>
       </c>
       <c r="B21" s="28" t="n">
@@ -5797,7 +5797,7 @@
         <v>0</v>
       </c>
       <c r="F21" s="29" t="n">
-        <v>1832.043468426193</v>
+        <v>1253.592714592957</v>
       </c>
       <c r="G21" s="30">
         <f>MIN(E21,Calculation!$B$3)*F21</f>
@@ -5862,23 +5862,23 @@
       <c r="Z21" s="28" t="n"/>
       <c r="AA21" s="28" t="n"/>
       <c r="AB21" s="28" t="n">
-        <v>212.7684182341731</v>
+        <v>0</v>
       </c>
       <c r="AC21" s="28" t="n">
-        <v>212.7684182341731</v>
+        <v>303.5887662103974</v>
       </c>
       <c r="AD21" s="33" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AE21" s="30">
         <f>MIN(AB21,Calculation!$B$3)*F21</f>
         <v/>
       </c>
       <c r="AF21" s="32" t="n">
-        <v>500.0000000000001</v>
+        <v>0</v>
       </c>
       <c r="AG21" s="34" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AH21" s="32" t="n">
         <v>0</v>
@@ -5930,7 +5930,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>002e15d9-b27f-4a99-b94d-703b11215eab</t>
+          <t>0078e0fc-2637-4256-9eb7-fbcc31d32e82</t>
         </is>
       </c>
       <c r="B22" s="28" t="n">
@@ -5944,7 +5944,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="29" t="n">
-        <v>816.216729440072</v>
+        <v>2252.313011387968</v>
       </c>
       <c r="G22" s="30">
         <f>MIN(E22,Calculation!$B$3)*F22</f>
@@ -6009,23 +6009,23 @@
       <c r="Z22" s="28" t="n"/>
       <c r="AA22" s="28" t="n"/>
       <c r="AB22" s="28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC22" s="28" t="n">
-        <v>252.3366353326147</v>
+        <v>424.0189758567727</v>
       </c>
       <c r="AD22" s="33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE22" s="30">
         <f>MIN(AB22,Calculation!$B$3)*F22</f>
         <v/>
       </c>
       <c r="AF22" s="32" t="n">
-        <v>0</v>
+        <v>500.0000000000001</v>
       </c>
       <c r="AG22" s="34" t="n">
-        <v>3</v>
+        <v>204</v>
       </c>
       <c r="AH22" s="32" t="n">
         <v>0</v>
@@ -6077,7 +6077,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>0078e0fc-2637-4256-9eb7-fbcc31d32e82</t>
+          <t>0120d782-7901-4838-9ae8-012ec8626771</t>
         </is>
       </c>
       <c r="B23" s="28" t="n">
@@ -6091,7 +6091,7 @@
         <v>0</v>
       </c>
       <c r="F23" s="29" t="n">
-        <v>1914.25567961288</v>
+        <v>1951.33667089501</v>
       </c>
       <c r="G23" s="30">
         <f>MIN(E23,Calculation!$B$3)*F23</f>
@@ -6156,23 +6156,23 @@
       <c r="Z23" s="28" t="n"/>
       <c r="AA23" s="28" t="n"/>
       <c r="AB23" s="28" t="n">
-        <v>9455.37551407438</v>
+        <v>0</v>
       </c>
       <c r="AC23" s="28" t="n">
-        <v>9455.37551407438</v>
+        <v>413.2027308032251</v>
       </c>
       <c r="AD23" s="33" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AE23" s="30">
         <f>MIN(AB23,Calculation!$B$3)*F23</f>
         <v/>
       </c>
       <c r="AF23" s="32" t="n">
-        <v>1500</v>
+        <v>200</v>
       </c>
       <c r="AG23" s="34" t="n">
-        <v>204</v>
+        <v>2</v>
       </c>
       <c r="AH23" s="32" t="n">
         <v>0</v>
@@ -6224,7 +6224,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>00ac4d7e-2245-4bfa-b36a-ef65994b6d02</t>
+          <t>0035a155-c4d3-4860-80e0-6c17481b3d61</t>
         </is>
       </c>
       <c r="B24" s="28" t="n">
@@ -6238,7 +6238,7 @@
         <v>0</v>
       </c>
       <c r="F24" s="29" t="n">
-        <v>1603.806741137101</v>
+        <v>2100.83789056557</v>
       </c>
       <c r="G24" s="30">
         <f>MIN(E24,Calculation!$B$3)*F24</f>
@@ -6303,23 +6303,23 @@
       <c r="Z24" s="28" t="n"/>
       <c r="AA24" s="28" t="n"/>
       <c r="AB24" s="28" t="n">
-        <v>2098.301874066376</v>
+        <v>0</v>
       </c>
       <c r="AC24" s="28" t="n">
-        <v>2098.301874066376</v>
+        <v>155.6974761971898</v>
       </c>
       <c r="AD24" s="33" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AE24" s="30">
         <f>MIN(AB24,Calculation!$B$3)*F24</f>
         <v/>
       </c>
       <c r="AF24" s="32" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="AG24" s="34" t="n">
-        <v>80</v>
+        <v>1</v>
       </c>
       <c r="AH24" s="32" t="n">
         <v>0</v>
@@ -6371,41 +6371,45 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>00224faa-3597-401e-b493-559fc185861b</t>
+          <t>0056ff07-ee70-495f-9a55-26d6aed9bd34</t>
         </is>
       </c>
       <c r="B25" s="28" t="n">
-        <v>0</v>
+        <v>13.66035760986725</v>
       </c>
       <c r="C25" s="28" t="n">
-        <v>0</v>
+        <v>14.62669252779978</v>
       </c>
       <c r="D25" s="28" t="n"/>
       <c r="E25" s="28" t="n">
-        <v>0</v>
+        <v>28.28705013766703</v>
       </c>
       <c r="F25" s="29" t="n">
-        <v>1142.349530467185</v>
+        <v>1348.528388619784</v>
       </c>
       <c r="G25" s="30">
         <f>MIN(E25,Calculation!$B$3)*F25</f>
         <v/>
       </c>
-      <c r="H25" s="4" t="inlineStr"/>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
       <c r="I25" s="31" t="n">
-        <v>0</v>
+        <v>1.75</v>
       </c>
       <c r="J25" s="28" t="n">
-        <v>0</v>
+        <v>11.52157565110756</v>
       </c>
       <c r="K25" s="32" t="n">
-        <v>0</v>
+        <v>18918.90478842935</v>
       </c>
       <c r="L25" s="28" t="n">
-        <v>0</v>
+        <v>25.42114382126615</v>
       </c>
       <c r="M25" s="32" t="n">
-        <v>0</v>
+        <v>3813.171573189923</v>
       </c>
       <c r="N25" s="30">
         <f>K25+M25</f>
@@ -6453,7 +6457,7 @@
         <v>0</v>
       </c>
       <c r="AC25" s="28" t="n">
-        <v>394.0728141999576</v>
+        <v>237.2603608836199</v>
       </c>
       <c r="AD25" s="33" t="n">
         <v>0</v>
@@ -6469,7 +6473,7 @@
         <v>1</v>
       </c>
       <c r="AH25" s="32" t="n">
-        <v>0</v>
+        <v>5355</v>
       </c>
       <c r="AI25" s="30">
         <f>N25+Y25+AF25+AH25</f>
@@ -6611,7 +6615,7 @@
     <row r="43">
       <c r="A43" s="35" t="inlineStr">
         <is>
-          <t>C1. Canterbury settled costs per property, $200 to $4,000 by damage state, in 2010/2011 dollars and NOT yet inflated. They exclude ILV and IFV, so they are the minor-damage tier only. The cap the state is compared against is the land rate over the whole insured area, because that is the scope those rates are per-property against.</t>
+          <t>C1. Canterbury settled costs per property, $200 to $4,000 by damage state, in 2010/2011 dollars and NOT yet inflated. They exclude ILV and IFV, so they are the minor-damage tier only. The cap the state is compared against is the land rate over the liquefied land: evacuated plus inundated, less the share of the evacuated assumed to overlap (L-44), no more than the insured area.</t>
         </is>
       </c>
     </row>

</xml_diff>